<commit_message>
Add Excel download endpoint
</commit_message>
<xml_diff>
--- a/data/generated_answers/rag_debug_logs.xlsx
+++ b/data/generated_answers/rag_debug_logs.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -3786,6 +3786,623 @@
         <v>15.4909815788269</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11T06:47:15.964358</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>What are the major departments under the MoD?</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document: Personnel Training and Professional Development in Armed Forces
+Similarity: 0.2583639621734619
+Text:
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academy (NDA): 4-year training for commission as officer
+        - Officers Training Academy (OTA): 49-week training for graduate officers
+        - Army Staff College: Senior officer strategy and leadership development
+        - War Colleges: Highest leve
+---------------------------------------
+Document: Personnel Training and Professional Development in Armed Forces
+Similarity: 0.24735736846923828
+Text:
+The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - 
+---------------------------------------
+Document: Joint Theatre Command Implementation Roadmap
+Similarity: 0.2378597855567932
+Text:
+Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Thea
+---------------------------------------
+Document: Counter-Terrorism Operations Manual and Best Practices
+Similarity: 0.23656296730041504
+Text:
+Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and N
+---------------------------------------
+Document: Counter-Terrorism Operations Manual and Best Practices
+Similarity: 0.23656296730041504
+Text:
+Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and N
+---------------------------------------
+Document: Defence Budget Allocation 2023-24: Analysis and Distribution
+Similarity: 0.2323359251022339
+Text:
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crore
+---------------------------------------
+Document: Defence Budget Allocation 2023-24: Analysis and Distribution
+Similarity: 0.22930198907852173
+Text:
+The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime
+---------------------------------------
+Document: Cyber Defence Architecture and National Digital Resilience Plan
+Similarity: 0.22827863693237305
+Text:
+Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems i
+---------------------------------------
+Document: Cyber Defence Architecture and National Digital Resilience Plan
+Similarity: 0.22827863693237305
+Text:
+Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems i
+---------------------------------------
+Document: Defence Procurement Policy 2023 - Strategic Framework
+Similarity: 0.22235876321792603
+Text:
+The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed </t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document 1: Unknown Document
+Content: 
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academy (NDA): 4-year training for commission as officer
+        - Officers Training Academy (OTA): 49-week training for graduate officers
+        - Army Staff College: Senior officer strategy and leadership development
+        - War Colleges: Highest level strategic and operational training
+        Enlisted Personnel Training:
+        - Basic Military Training Centers: 6-12 week initial training
+        - Trade-specific Training: Pilots, engineers, medical, signals, etc.
+        - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs
+        - Continuing Education: Annual refresher courses on latest tactics and technology
+        Technology Training:
+        - Pilot Training on Rafale, Tejas, and other aircraft
+        - Submarine Crew Training: Advanced underwater warfare tactics
+        - Cyber Warfare Training: Defense against digital threats
+        - Artificial Intelligence Applications: Machine learning and autonomous systems
+        - Unmanned Systems: Drone and robot operation and maintenance
+        International Exchange:
+        - Training exchanges with allied nations (USA, UK, France, Israel)
+        - Joint exercises providing real-world training scenarios
+        - Instructor attachments at foreign military academies
+        - Participation in international military competitions
+        Standards and Evaluation:
+        - Rigorous evaluation standards ensuring combat readiness
+        - Competency-based assessment of all critical skills
+        - Regular audits of training effectiveness
+        - Feedback loops for continuous improvement of curriculum
+Relevance: 25.8%
+---
+Document 2: Personnel Training and Professional Development in Armed Forces
+Content: The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - Basic Military Training Centers: 6-12 week initial training - Trade-specific Training: Pilots, engineers, medical, signals, etc - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs - Continuing Education: Annual refresher courses on latest tactics and technology Technology Training: - Pilot Training on Rafale, Tejas, and other aircraft - Submarine Crew Training: Advanced underwater warfare tactics - Cyber Warfare Training: Defense against digital threats - Artificial Intelligence Applications: Machine learning and autonomous systems - Unmanned Systems: Drone and robot operation and maintenance International Exchange: - Training exchanges with allied nations (USA, UK, France, Israel) - Joint exercises providing real-world training scenarios - Instructor attachments at foreign military academies - Participation in international military competitions Standards and Evaluation: - Rigorous evaluation standards ensuring combat readiness - Competency-based assessment of all critical skills - Regular audits of training effectiveness - Feedback loops for continuous improvement of curriculum
+Relevance: 24.7%
+---
+Document 3: Joint Theatre Command Implementation Roadmap
+Content: Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Theatre (Indian Ocean), Cyber Theatre (digital warfare operations), Space Theatre (satellite operations and space defence) Expected efficiency gains from unification: 15-20% reduction in administrative overhead and redundant support structures, faster decision-making cycles through simplified command chains, improved inter-service coordination eliminating compartmentalization, and better resource optimization Transition timeline structured in three phases: Phase 1 (2024-25) establishes new command structures with compatible organizational frameworks; Phase 2 (2025-26) implements resource consolidation with integrated logistics and personnel management; Phase 3 (2026-27) achieves full operationalization with theatre-level integrated exercises demonstrating seamless inter-service coordination Risk mitigation strategies address potential institutional disruption through: smooth transition protocols minimizing operational gaps, comprehensive training programs for officers and support staff adapting to new command structures, maintenance of continuity during transition period, and retention mechanisms for experienced personnel Technology integration includes unified command and control systems, real-time data sharing across services, and AI-based decision support systems providing situational assessment and recommendation synthesis Performance metrics for successful theatre command implementation include reduced decision-making timelines, improved operational effectiveness metrics, enhanced inter-service coordination demonstrated through joint exercises, and cost optimization targets The transformation represents major institutional change requiring sustained commitment from military leadership, government support, and international partnerships with allied nations having similar structures
+Relevance: 23.8%
+---
+Document 4: Counter-Terrorism Operations Manual and Best Practices
+Content: Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and Northeast with elevation challenges, urban environments in metro areas with civilian density considerations, and riverine operations in wetland areas Training requirements specify 500+ hours for frontline operators covering weapons handling, tactical movement, hostage rescue techniques, and cultural awareness Support personnel require 200+ hours training in logistics, communications, and medical support Technology deployment includes unmanned aerial vehicles for surveillance, secure communication systems with encryption, and real-time intelligence fusion systems Success metrics include 95%+ mission completion rate, civilian casualty minimization, and efficiency in intelligence gathering Specialized operations training covers mountaineering and altitude acclimatization, urban close-quarter combat, helicopter insertion techniques, and underwater operations Equipment standards specify precision rifles, advanced body armor, night vision systems, and thermal imaging capabilities Command and control protocols establish clear chains of authority, abort decision criteria, and coordination procedures After-action reviews systematically capture lessons learned and identify capability improvements International training exchanges with allied nations provide exposure to different operational approaches and best practices Counter-terrorism doctrine continues evolving based on threat analysis and emerging tactics
+Relevance: 23.7%
+---
+Document 5: Counter-Terrorism Operations Manual and Best Practices
+Content: Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and Northeast with elevation challenges, urban environments in metro areas with civilian density considerations, and riverine operations in wetland areas Training requirements specify 500+ hours for frontline operators covering weapons handling, tactical movement, hostage rescue techniques, and cultural awareness Support personnel require 200+ hours training in logistics, communications, and medical support Technology deployment includes unmanned aerial vehicles for surveillance, secure communication systems with encryption, and real-time intelligence fusion systems Success metrics include 95%+ mission completion rate, civilian casualty minimization, and efficiency in intelligence gathering Specialized operations training covers mountaineering and altitude acclimatization, urban close-quarter combat, helicopter insertion techniques, and underwater operations Equipment standards specify precision rifles, advanced body armor, night vision systems, and thermal imaging capabilities Command and control protocols establish clear chains of authority, abort decision criteria, and coordination procedures After-action reviews systematically capture lessons learned and identify capability improvements International training exchanges with allied nations provide exposure to different operational approaches and best practices Counter-terrorism doctrine continues evolving based on threat analysis and emerging tactics
+Relevance: 23.7%
+---
+Document 6: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 23.2%
+---
+Document 7: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 22.9%
+---
+Document 8: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 22.8%
+---
+Document 9: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 22.8%
+---
+Document 10: Defence Procurement Policy 2023 - Strategic Framework
+Content: The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems 4 Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts 5 Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, Contract Negotiation, and Implementation with quarterly reviews All decisions are documented for transparency Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements
+Relevance: 22.2%
+---
+Document 11: Border Management and Coastal Security Operations Manual
+Content: Standard procedures for comprehensive management of 15,106 kilometers of land border and 7,517 kilometers of coastline Surveillance infrastructure encompasses 2,500+ surveillance cameras, comprehensive sensor networks, and real-time satellite imagery feeds Personnel deployment across all borders totals 500,000+ trained personnel providing continuous presence and rapid response capability Technology integration includes automated threat detection systems, unmanned drone patrols with extended flight endurance, and sensor fusion systems correlating multiple data sources for threat identification Coordination mechanisms link Border Security Force, Coast Guard, state police, and military units through unified command structures Cross-border incident protocols establish communication channels, rules for engagement, de-escalation procedures, and escalation pathways for different threat levels Coastal security operations deploy 500+ interceptor boats, naval vessels with advanced weapons systems, and aircraft providing surveillance and rapid response Infrastructure security measures protect strategic ports, naval facilities, and critical communication installations from sabotage and terrorism Personnel training covers border patrolling techniques, threat recognition protocols, communication procedures, and emergency response Environmental monitoring identifies unusual activities including smuggling operations, infiltration attempts, and illegal maritime activities Technology provides early warning of aerial threats, vehicular movement detection, and precision identification of crossing points Intelligence sharing with international partners including Bangladesh, Myanmar, and Pakistan reduces transnational criminal activity Statistics tracking monitors penetration attempts, interdiction rates, and incident patterns informing continuous operational improvements
+Relevance: 21.2%
+---
+Document 12: Border Management and Coastal Security Operations Manual
+Content: Standard procedures for comprehensive management of 15,106 kilometers of land border and 7,517 kilometers of coastline Surveillance infrastructure encompasses 2,500+ surveillance cameras, comprehensive sensor networks, and real-time satellite imagery feeds Personnel deployment across all borders totals 500,000+ trained personnel providing continuous presence and rapid response capability Technology integration includes automated threat detection systems, unmanned drone patrols with extended flight endurance, and sensor fusion systems correlating multiple data sources for threat identification Coordination mechanisms link Border Security Force, Coast Guard, state police, and military units through unified command structures Cross-border incident protocols establish communication channels, rules for engagement, de-escalation procedures, and escalation pathways for different threat levels Coastal security operations deploy 500+ interceptor boats, naval vessels with advanced weapons systems, and aircraft providing surveillance and rapid response Infrastructure security measures protect strategic ports, naval facilities, and critical communication installations from sabotage and terrorism Personnel training covers border patrolling techniques, threat recognition protocols, communication procedures, and emergency response Environmental monitoring identifies unusual activities including smuggling operations, infiltration attempts, and illegal maritime activities Technology provides early warning of aerial threats, vehicular movement detection, and precision identification of crossing points Intelligence sharing with international partners including Bangladesh, Myanmar, and Pakistan reduces transnational criminal activity Statistics tracking monitors penetration attempts, interdiction rates, and incident patterns informing continuous operational improvements
+Relevance: 21.2%
+---
+Document 13: Veterans' Rehabilitation and Post-Service Support Program
+Content: The Veterans' Rehabilitation and Post-Service Support Program ensures dignified rehabilitation and reintegration of retired military personnel into civilian society Healthcare Services: - Free medical treatment for service-connected disabilities at defense hospitals - ECHS (Ex-Servicemen Contribution Health Scheme): Pan-India medical network coverage - Mental health support and PTSD counseling for combat trauma - Geriatric care centers for aging veterans and their dependents - Artificial limbs and prosthetics for disabled veterans Financial Support: - Disability pensions based on extent of disability (0-100%) - Pension reviews every 3 years with inflation adjustments - One-time rehabilitation grant for economically backward veterans - Interest-free loans for business startup and self-employment - Housing assistance and concessional housing schemes Employment Assistance: - Priority employment in civilian government and PSU jobs - Skill development courses in high-demand sectors - Self-employment training and business mentoring - Job placement assistance through employment fairs - Reservation in police forces and paramilitary organizations Education Support: - Scholarship programs for children of war casualties - Concessional admission to defense institutes and universities - Vocational training in engineering and trades - Adult literacy programs for less educated veterans Community Integration: - Veteran peer support groups and networking organizations - Recreational facilities and sports programs - Cultural programs and ceremonial recognition events - Grievance redressal mechanism for benefits disputes
+Relevance: 21.1%
+---
+Document 14: Unknown Document
+Content: 
+        The Veterans' Rehabilitation and Post-Service Support Program ensures dignified rehabilitation 
+        and reintegration of retired military personnel into civilian society.
+        Healthcare Services:
+        - Free medical treatment for service-connected disabilities at defense hospitals
+        - ECHS (Ex-Servicemen Contribution Health Scheme): Pan-India medical network coverage
+        - Mental health support and PTSD counseling for combat trauma
+        - Geriatric care centers for aging veterans and their dependents
+        - Artificial limbs and prosthetics for disabled veterans
+        Financial Support:
+        - Disability pensions based on extent of disability (0-100%)
+        - Pension reviews every 3 years with inflation adjustments
+        - One-time rehabilitation grant for economically backward veterans
+        - Interest-free loans for business startup and self-employment
+        - Housing assistance and concessional housing schemes
+        Employment Assistance:
+        - Priority employment in civilian government and PSU jobs
+        - Skill development courses in high-demand sectors
+        - Self-employment training and business mentoring
+        - Job placement assistance through employment fairs
+        - Reservation in police forces and paramilitary organizations
+        Education Support:
+        - Scholarship programs for children of war casualties
+        - Concessional admission to defense institutes and universities
+        - Vocational training in engineering and trades
+        - Adult literacy programs for less educated veterans
+        Community Integration:
+        - Veteran peer support groups and networking organizations
+        - Recreational facilities and sports programs
+        - Cultural programs and ceremonial recognition events
+        - Grievance redressal mechanism for benefits disputes
+Relevance: 21.1%
+---
+Document 15: Unknown Document
+Content: 
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include:
+        1. Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content.
+        2. Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems.
+        3. FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems.
+        4. Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts.
+        5. Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years.
+        The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, 
+        Contract Negotiation, and Implementation with quarterly reviews. All decisions are documented for transparency.
+        Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development.
+        The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements.
+Relevance: 20.4%
+</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a Defence Intelligence Assistant.
+DOCUMENTS:
+Document 1: Unknown Document
+Content: 
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academy (NDA): 4-year training for commission as officer
+        - Officers Training Academy (OTA): 49-week training for graduate officers
+        - Army Staff College: Senior officer strategy and leadership development
+        - War Colleges: Highest level strategic and operational training
+        Enlisted Personnel Training:
+        - Basic Military Training Centers: 6-12 week initial training
+        - Trade-specific Training: Pilots, engineers, medical, signals, etc.
+        - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs
+        - Continuing Education: Annual refresher courses on latest tactics and technology
+        Technology Training:
+        - Pilot Training on Rafale, Tejas, and other aircraft
+        - Submarine Crew Training: Advanced underwater warfare tactics
+        - Cyber Warfare Training: Defense against digital threats
+        - Artificial Intelligence Applications: Machine learning and autonomous systems
+        - Unmanned Systems: Drone and robot operation and maintenance
+        International Exchange:
+        - Training exchanges with allied nations (USA, UK, France, Israel)
+        - Joint exercises providing real-world training scenarios
+        - Instructor attachments at foreign military academies
+        - Participation in international military competitions
+        Standards and Evaluation:
+        - Rigorous evaluation standards ensuring combat readiness
+        - Competency-based assessment of all critical skills
+        - Regular audits of training effectiveness
+        - Feedback loops for continuous improvement of curriculum
+Relevance: 25.8%
+---
+Document 2: Personnel Training and Professional Development in Armed Forces
+Content: The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - Basic Military Training Centers: 6-12 week initial training - Trade-specific Training: Pilots, engineers, medical, signals, etc - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs - Continuing Education: Annual refresher courses on latest tactics and technology Technology Training: - Pilot Training on Rafale, Tejas, and other aircraft - Submarine Crew Training: Advanced underwater warfare tactics - Cyber Warfare Training: Defense against digital threats - Artificial Intelligence Applications: Machine learning and autonomous systems - Unmanned Systems: Drone and robot operation and maintenance International Exchange: - Training exchanges with allied nations (USA, UK, France, Israel) - Joint exercises providing real-world training scenarios - Instructor attachments at foreign military academies - Participation in international military competitions Standards and Evaluation: - Rigorous evaluation standards ensuring combat readiness - Competency-based assessment of all critical skills - Regular audits of training effectiveness - Feedback loops for continuous improvement of curriculum
+Relevance: 24.7%
+---
+Document 3: Joint Theatre Command Implementation Roadmap
+Content: Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Theatre (Indian Ocean), Cyber Theatre (digital warfare operations), Space Theatre (satellite operations and space defence) Expected efficiency gains from unification: 15-20% reduction in administrative overhead and redundant support structures, faster decision-making cycles through simplified command chains, improved inter-service coordination eliminating compartmentalization, and better resource optimization Transition timeline structured in three phases: Phase 1 (2024-25) establishes new command structures with compatible organizational frameworks; Phase 2 (2025-26) implements resource consolidation with integrated logistics and personnel management; Phase 3 (2026-27) achieves full operationalization with theatre-level integrated exercises demonstrating seamless inter-service coordination Risk mitigation strategies address potential institutional disruption through: smooth transition protocols minimizing operational gaps, comprehensive training programs for officers and support staff adapting to new command structures, maintenance of continuity during transition period, and retention mechanisms for experienced personnel Technology integration includes unified command and control systems, real-time data sharing across services, and AI-based decision support systems providing situational assessment and recommendation synthesis Performance metrics for successful theatre command implementation include reduced decision-making timelines, improved operational effectiveness metrics, enhanced inter-service coordination demonstrated through joint exercises, and cost optimization targets The transformation represents major institutional change requiring sustained commitment from military leadership, government support, and international partnerships with allied nations having similar structures
+Relevance: 23.8%
+---
+Document 4: Counter-Terrorism Operations Manual and Best Practices
+Content: Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and Northeast with elevation challenges, urban environments in metro areas with civilian density considerations, and riverine operations in wetland areas Training requirements specify 500+ hours for frontline operators covering weapons handling, tactical movement, hostage rescue techniques, and cultural awareness Support personnel require 200+ hours training in logistics, communications, and medical support Technology deployment includes unmanned aerial vehicles for surveillance, secure communication systems with encryption, and real-time intelligence fusion systems Success metrics include 95%+ mission completion rate, civilian casualty minimization, and efficiency in intelligence gathering Specialized operations training covers mountaineering and altitude acclimatization, urban close-quarter combat, helicopter insertion techniques, and underwater operations Equipment standards specify precision rifles, advanced body armor, night vision systems, and thermal imaging capabilities Command and control protocols establish clear chains of authority, abort decision criteria, and coordination procedures After-action reviews systematically capture lessons learned and identify capability improvements International training exchanges with allied nations provide exposure to different operational approaches and best practices Counter-terrorism doctrine continues evolving based on threat analysis and emerging tactics
+Relevance: 23.7%
+---
+Document 5: Counter-Terrorism Operations Manual and Best Practices
+Content: Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and Northeast with elevation challenges, urban environments in metro areas with civilian density considerations, and riverine operations in wetland areas Training requirements specify 500+ hours for frontline operators covering weapons handling, tactical movement, hostage rescue techniques, and cultural awareness Support personnel require 200+ hours training in logistics, communications, and medical support Technology deployment includes unmanned aerial vehicles for surveillance, secure communication systems with encryption, and real-time intelligence fusion systems Success metrics include 95%+ mission completion rate, civilian casualty minimization, and efficiency in intelligence gathering Specialized operations training covers mountaineering and altitude acclimatization, urban close-quarter combat, helicopter insertion techniques, and underwater operations Equipment standards specify precision rifles, advanced body armor, night vision systems, and thermal imaging capabilities Command and control protocols establish clear chains of authority, abort decision criteria, and coordination procedures After-action reviews systematically capture lessons learned and identify capability improvements International training exchanges with allied nations provide exposure to different operational approaches and best practices Counter-terrorism doctrine continues evolving based on threat analysis and emerging tactics
+Relevance: 23.7%
+---
+Document 6: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 23.2%
+---
+Document 7: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 22.9%
+---
+Document 8: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 22.8%
+---
+Document 9: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 22.8%
+---
+Document 10: Defence Procurement Policy 2023 - Strategic Framework
+Content: The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems 4 Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts 5 Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, Contract Negotiation, and Implementation with quarterly reviews All decisions are documented for transparency Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements
+Relevance: 22.2%
+---
+Document 11: Border Management and Coastal Security Operations Manual
+Content: Standard procedures for comprehensive management of 15,106 kilometers of land border and 7,517 kilometers of coastline Surveillance infrastructure encompasses 2,500+ surveillance cameras, comprehensive sensor networks, and real-time satellite imagery feeds Personnel deployment across all borders totals 500,000+ trained personnel providing continuous presence and rapid response capability Technology integration includes automated threat detection systems, unmanned drone patrols with extended flight endurance, and sensor fusion systems correlating multiple data sources for threat identification Coordination mechanisms link Border Security Force, Coast Guard, state police, and military units through unified command structures Cross-border incident protocols establish communication channels, rules for engagement, de-escalation procedures, and escalation pathways for different threat levels Coastal security operations deploy 500+ interceptor boats, naval vessels with advanced weapons systems, and aircraft providing surveillance and rapid response Infrastructure security measures protect strategic ports, naval facilities, and critical communication installations from sabotage and terrorism Personnel training covers border patrolling techniques, threat recognition protocols, communication procedures, and emergency response Environmental monitoring identifies unusual activities including smuggling operations, infiltration attempts, and illegal maritime activities Technology provides early warning of aerial threats, vehicular movement detection, and precision identification of crossing points Intelligence sharing with international partners including Bangladesh, Myanmar, and Pakistan reduces transnational criminal activity Statistics tracking monitors penetration attempts, interdiction rates, and incident patterns informing continuous operational improvements
+Relevance: 21.2%
+---
+Document 12: Border Management and Coastal Security Operations Manual
+Content: Standard procedures for comprehensive management of 15,106 kilometers of land border and 7,517 kilometers of coastline Surveillance infrastructure encompasses 2,500+ surveillance cameras, comprehensive sensor networks, and real-time satellite imagery feeds Personnel deployment across all borders totals 500,000+ trained personnel providing continuous presence and rapid response capability Technology integration includes automated threat detection systems, unmanned drone patrols with extended flight endurance, and sensor fusion systems correlating multiple data sources for threat identification Coordination mechanisms link Border Security Force, Coast Guard, state police, and military units through unified command structures Cross-border incident protocols establish communication channels, rules for engagement, de-escalation procedures, and escalation pathways for different threat levels Coastal security operations deploy 500+ interceptor boats, naval vessels with advanced weapons systems, and aircraft providing surveillance and rapid response Infrastructure security measures protect strategic ports, naval facilities, and critical communication installations from sabotage and terrorism Personnel training covers border patrolling techniques, threat recognition protocols, communication procedures, and emergency response Environmental monitoring identifies unusual activities including smuggling operations, infiltration attempts, and illegal maritime activities Technology provides early warning of aerial threats, vehicular movement detection, and precision identification of crossing points Intelligence sharing with international partners including Bangladesh, Myanmar, and Pakistan reduces transnational criminal activity Statistics tracking monitors penetration attempts, interdiction rates, and incident patterns informing continuous operational improvements
+Relevance: 21.2%
+---
+Document 13: Veterans' Rehabilitation and Post-Service Support Program
+Content: The Veterans' Rehabilitation and Post-Service Support Program ensures dignified rehabilitation and reintegration of retired military personnel into civilian society Healthcare Services: - Free medical treatment for service-connected disabilities at defense hospitals - ECHS (Ex-Servicemen Contribution Health Scheme): Pan-India medical network coverage - Mental health support and PTSD counseling for combat trauma - Geriatric care centers for aging veterans and their dependents - Artificial limbs and prosthetics for disabled veterans Financial Support: - Disability pensions based on extent of disability (0-100%) - Pension reviews every 3 years with inflation adjustments - One-time rehabilitation grant for economically backward veterans - Interest-free loans for business startup and self-employment - Housing assistance and concessional housing schemes Employment Assistance: - Priority employment in civilian government and PSU jobs - Skill development courses in high-demand sectors - Self-employment training and business mentoring - Job placement assistance through employment fairs - Reservation in police forces and paramilitary organizations Education Support: - Scholarship programs for children of war casualties - Concessional admission to defense institutes and universities - Vocational training in engineering and trades - Adult literacy programs for less educated veterans Community Integration: - Veteran peer support groups and networking organizations - Recreational facilities and sports programs - Cultural programs and ceremonial recognition events - Grievance redressal mechanism for benefits disputes
+Relevance: 21.1%
+---
+Document 14: Unknown Document
+Content: 
+        The Veterans' Rehabilitation and Post-Service Support Program ensures dignified rehabilitation 
+        and reintegration of retired military personnel into civilian society.
+        Healthcare Services:
+        - Free medical treatment for service-connected disabilities at defense hospitals
+        - ECHS (Ex-Servicemen Contribution Health Scheme): Pan-India medical network coverage
+        - Mental health support and PTSD counseling for combat trauma
+        - Geriatric care centers for aging veterans and their dependents
+        - Artificial limbs and prosthetics for disabled veterans
+        Financial Support:
+        - Disability pensions based on extent of disability (0-100%)
+        - Pension reviews every 3 years with inflation adjustments
+        - One-time rehabilitation grant for economically backward veterans
+        - Interest-free loans for business startup and self-employment
+        - Housing assistance and concessional housing schemes
+        Employment Assistance:
+        - Priority employment in civilian government and PSU jobs
+        - Skill development courses in high-demand sectors
+        - Self-employment training and business mentoring
+        - Job placement assistance through employment fairs
+        - Reservation in police forces and paramilitary organizations
+        Education Support:
+        - Scholarship programs for children of war casualties
+        - Concessional admission to defense institutes and universities
+        - Vocational training in engineering and trades
+        - Adult literacy programs for less educated veterans
+        Community Integration:
+        - Veteran peer support groups and networking organizations
+        - Recreational facilities and sports programs
+        - Cultural programs and ceremonial recognition events
+        - Grievance redressal mechanism for benefits disputes
+Relevance: 21.1%
+---
+Document 15: Unknown Document
+Content: 
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include:
+        1. Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content.
+        2. Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems.
+        3. FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems.
+        4. Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts.
+        5. Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years.
+        The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, 
+        Contract Negotiation, and Implementation with quarterly reviews. All decisions are documented for transparency.
+        Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development.
+        The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements.
+Relevance: 20.4%
+QUESTION:
+What are the major departments under the MoD?
+ANSWER:
+</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>The context provided does not explicitly mention the major departments under the Ministry of Defence (MoD). However, based on the information available in the documents, we can infer the existence of the following departments or branches:
+1. Department of Military Affairs: Although not directly mentioned, the context suggests the presence of departments responsible for military affairs, such as training, operations, and personnel management.
+2. Department of Defence Production: The Defence Procurement Policy 2023 (Document 10 and Document 15) implies the existence of a department responsible for defence production, acquisition, and procurement.
+3. Department of Ex-Servicemen Welfare: The Veterans' Rehabilitation and Post-Service Support Program (Document 13 and Document 14) suggests a department focused on the welfare of ex-servicemen and veterans.
+4. Department of Defence Finance: The Defence Budget Allocation 2023-24 (Document 6 and Document 7) implies the presence of a department responsible for managing the defence budget and finances.
+5. Department of Border Management: The Border Management and Coastal Security Operations Manual (Document 11 and Document 12) suggests a department responsible for border management and coastal security.
+Please note that these inferences are based on the context provided and may not be an exhaustive list of all departments under the MoD. For a comprehensive and accurate answer, it is recommended to consult official government sources or the Ministry of Defence's official website.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Based on the retrieved documents:
+1. From 'Personnel Training and Professional Development in Armed Forces' (confidence: 25.8%):
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academ...
+2. From 'Document' (confidence: 24.7%):
+   The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as o...
+3. From 'Document' (confidence: 23.8%):
+   Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined c...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>EXECUTIVE SUMMARY:
+Question: What are the major departments under the MoD?
+Overview:
+This report synthesizes intelligence from three independent model analyses and a fallback summary. It highlights common findings, discrepancies, and operational implications.
+Combined Analysis:
+Gemini Analysis:
+No Gemini output available.
+Groq Analysis:
+The context provided does not explicitly mention the major departments under the Ministry of Defence (MoD). However, based on the information available in the documents, we can infer the existence of the following departments or branches:
+1. Department of Military Affairs: Although not directly mentioned, the context suggests the presence of departments responsible for military affairs, such as training, operations, and personnel management.
+2. Department of Defence Production: The Defence Procurement Policy 2023 (Document 10 and Document 15) implies the existence of a department responsible for defence production, acquisition, and procurement.
+3. Department of Ex-Servicemen Welfare: The Veterans' Rehabilitation and Post-Service Support Program (Document 13 and Document 14) suggests a department focused on the welfare of ex-servicemen and veterans.
+4. Department of Defence Finance: The Defence Budget Allocation 2023-24 (Document 6 and Document 7) implies the presence of a department responsible for managing the defence budget and finances.
+5. Department of Border Management: The Border Management and Coastal Security Operations Manual (Document 11 and Document 12) suggests a department responsible for border management and coastal security.
+Please note that these inferences are based on the context provided and may not be an exhaustive list of all departments under the MoD. For a comprehensive and accurate answer, it is recommended to consult official government sources or the Ministry of Defence's official website.
+Grok Analysis:
+No Grok output available.
+Fallback Analysis:
+Based on the retrieved documents:
+1. From 'Personnel Training and Professional Development in Armed Forces' (confidence: 25.8%):
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academ...
+2. From 'Document' (confidence: 24.7%):
+   The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as o...
+3. From 'Document' (confidence: 23.8%):
+   Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined c...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.
+Key Findings:
+- Groq: The context provided does not explicitly mention the major departments under the Ministry of Defence (MoD). However, based on the information available in the documents, we can infer the existence of the following departments or branches:...
+Detailed Analysis:
+Gemini Analysis:
+No Gemini output available.
+Groq Analysis:
+The context provided does not explicitly mention the major departments under the Ministry of Defence (MoD). However, based on the information available in the documents, we can infer the existence of the following departments or branches:
+1. Department of Military Affairs: Although not directly mentioned, the context suggests the presence of departments responsible for military affairs, such as training, operations, and personnel management.
+2. Department of Defence Production: The Defence Procurement Policy 2023 (Document 10 and Document 15) implies the existence of a department responsible for defence production, acquisition, and procurement.
+3. Department of Ex-Servicemen Welfare: The Veterans' Rehabilitation and Post-Service Support Program (Document 13 and Document 14) suggests a department focused on the welfare of ex-servicemen and veterans.
+4. Department of Defence Finance: The Defence Budget Allocation 2023-24 (Document 6 and Document 7) implies the presence of a department responsible for managing the defence budget and finances.
+5. Department of Border Management: The Border Management and Coastal Security Operations Manual (Document 11 and Document 12) suggests a department responsible for border management and coastal security.
+Please note that these inferences are based on the context provided and may not be an exhaustive list of all departments under the MoD. For a comprehensive and accurate answer, it is recommended to consult official government sources or the Ministry of Defence's official website.
+Grok Analysis:
+No Grok output available.
+Fallback Analysis:
+Based on the retrieved documents:
+1. From 'Personnel Training and Professional Development in Armed Forces' (confidence: 25.8%):
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academ...
+2. From 'Document' (confidence: 24.7%):
+   The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as o...
+3. From 'Document' (confidence: 23.8%):
+   Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined c...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.
+Retrieved Context and Sources:
+Document 1: Unknown Document
+Content: 
+        The Armed Forces training and development program ensures that military personnel are equipped with 
+        cutting-edge knowledge and skills for modern warfare.
+        Officer Training Academies:
+        - National Defence Academy (NDA): 4-year training for commission as officer
+        - Officers Training Academy (OTA): 49-week training for graduate officers
+        - Army Staff College: Senior officer strategy and leadership development
+        - War Colleges: Highest level strategic and operational training
+        Enlisted Personnel Training:
+        - Basic Military Training Centers: 6-12 week initial training
+        - Trade-specific Training: Pilots, engineers, medical, signals, etc.
+        - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs
+        - Continuing Education: Annual refresher courses on latest tactics and technology
+        Technology Training:
+        - Pilot Training on Rafale, Tejas, and other aircraft
+        - Submarine Crew Training: Advanced underwater warfare tactics
+        - Cyber Warfare Training: Defense against digital threats
+        - Artificial Intelligence Applications: Machine learning and autonomous systems
+        - Unmanned Systems: Drone and robot operation and maintenance
+        International Exchange:
+        - Training exchanges with allied nations (USA, UK, France, Israel)
+        - Joint exercises providing real-world training scenarios
+        - Instructor attachments at foreign military academies
+        - Participation in international military competitions
+        Standards and Evaluation:
+        - Rigorous evaluation standards ensuring combat readiness
+        - Competency-based assessment of all critical skills
+        - Regular audits of training effectiveness
+        - Feedback loops for continuous improvement of curriculum
+Relevance: 25.8%
+---
+Document 2: Personnel Training and Professional Development in Armed Forces
+Content: The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - Basic Military Training Centers: 6-12 week initial training - Trade-specific Training: Pilots, engineers, medical, signals, etc - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs - Continuing Education: Annual refresher courses on latest tactics and technology Technology Training: - Pilot Training on Rafale, Tejas, and other aircraft - Submarine Crew Training: Advanced underwater warfare tactics - Cyber Warfare Training: Defense against digital threats - Artificial Intelligence Applications: Machine learning and autonomous systems - Unmanned Systems: Drone and robot operation and maintenance International Exchange: - Training exchanges with allied nations (USA, UK, France, Israel) - Joint exercises providing real-world training scenarios - Instructor attachments at foreign military academies - Participation in international military competitions Standards and Evaluation: - Rigorous evaluation standards ensuring combat readiness - Competency-based assessment of all critical skills - Regular audits of training effectiveness - Feedback loops for continuous improvement of curriculum
+Relevance: 24.7%
+---
+Document 3: Joint Theatre Command Implementation Roadmap
+Content: Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Theatre (Indian Ocean), Cyber Theatre (digital warfare operations), Space Theatre (satellite operations and space defence) Expected efficiency gains from unification: 15-20% reduction in administrative overhead and redundant support structures, faster decision-making cycles through simplified command chains, improved inter-service coordination eliminating compartmentalization, and better resource optimization Transition timeline structured in three phases: Phase 1 (2024-25) establishes new command structures with compatible organizational frameworks; Phase 2 (2025-26) implements resource consolidation with integrated logistics and personnel management; Phase 3 (2026-27) achieves full operationalization with theatre-level integrated exercises demonstrating seamless inter-service coordination Risk mitigation strategies address potential institutional disruption through: smooth transition protocols minimizing operational gaps, comprehensive training programs for officers and support staff adapting to new command structures, maintenance of continuity during transition period, and retention mechanisms for experienced personnel Technology integration includes unified command and control systems, real-time data sharing across services, and AI-based decision support systems providing situational assessment and recommendation synthesis Performance metrics for successful theatre command implementation include reduced decision-making timelines, improved operational effectiveness metrics, enhanced inter-service coordination demonstrated through joint exercises, and cost optimization targets The transformation represents major institutional change requiring sustained commitment from military leadership, government support, and international partnerships with allied nations having similar structures
+Relevance: 23.8%
+---
+Document 4: Counter-Terrorism Operations Manual and Best Practices
+Content: Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and Northeast with elevation challenges, urban environments in metro areas with civilian density considerations, and riverine operations in wetland areas Training requirements specify 500+ hours for frontline operators covering weapons handling, tactical movement, hostage rescue techniques, and cultural awareness Support personnel require 200+ hours training in logistics, communications, and medical support Technology deployment includes unmanned aerial vehicles for surveillance, secure communication systems with encryption, and real-time intelligence fusion systems Success metrics include 95%+ mission completion rate, civilian casualty minimization, and efficiency in intelligence gathering Specialized operations training covers mountaineering and altitude acclimatization, urban close-quarter combat, helicopter insertion techniques, and underwater operations Equipment standards specify precision rifles, advanced body armor, night vision systems, and thermal imaging capabilities Command and control protocols establish clear chains of authority, abort decision criteria, and coordination procedures After-action reviews systematically capture lessons learned and identify capability improvements International training exchanges with allied nations provide exposure to different operational approaches and best practices Counter-terrorism doctrine continues evolving based on threat analysis and emerging tactics
+Relevance: 23.7%
+---
+Document 5: Counter-Terrorism Operations Manual and Best Practices
+Content: Comprehensive operational guidelines for counter-terrorism missions across diverse geographical and operational contexts Integration of intelligence, surveillance, and reconnaissance capabilities with tactical operations provides real-time situational awareness Rules of engagement emphasizing civilian protection and proportionality ensure operations comply with international humanitarian law Standard operating procedures adapted for different terrain types: mountainous regions like Kashmir and Northeast with elevation challenges, urban environments in metro areas with civilian density considerations, and riverine operations in wetland areas Training requirements specify 500+ hours for frontline operators covering weapons handling, tactical movement, hostage rescue techniques, and cultural awareness Support personnel require 200+ hours training in logistics, communications, and medical support Technology deployment includes unmanned aerial vehicles for surveillance, secure communication systems with encryption, and real-time intelligence fusion systems Success metrics include 95%+ mission completion rate, civilian casualty minimization, and efficiency in intelligence gathering Specialized operations training covers mountaineering and altitude acclimatization, urban close-quarter combat, helicopter insertion techniques, and underwater operations Equipment standards specify precision rifles, advanced body armor, night vision systems, and thermal imaging capabilities Command and control protocols establish clear chains of authority, abort decision criteria, and coordination procedures After-action reviews systematically capture lessons learned and identify capability improvements International training exchanges with allied nations provide exposure to different operational approaches and best practices Counter-terrorism doctrine continues evolving based on threat analysis and emerging tactics
+Relevance: 23.7%
+---
+Document 6: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 23.2%
+---
+Document 7: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 22.9%
+---
+Document 8: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 22.8%
+---
+Document 9: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 22.8%
+---
+Document 10: Defence Procurement Policy 2023 - Strategic Framework
+Content: The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems 4 Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts 5 Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, Contract Negotiation, and Implementation with quarterly reviews All decisions are documented for transparency Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements
+Relevance: 22.2%
+---
+Document 11: Border Management and Coastal Security Operations Manual
+Content: Standard procedures for comprehensive management of 15,106 kilometers of land border and 7,517 kilometers of coastline Surveillance infrastructure encompasses 2,500+ surveillance cameras, comprehensive sensor networks, and real-time satellite imagery feeds Personnel deployment across all borders totals 500,000+ trained personnel providing continuous presence and rapid response capability Technology integration includes automated threat detection systems, unmanned drone patrols with extended flight endurance, and sensor fusion systems correlating multiple data sources for threat identification Coordination mechanisms link Border Security Force, Coast Guard, state police, and military units through unified command structures Cross-border incident protocols establish communication channels, rules for engagement, de-escalation procedures, and escalation pathways for different threat levels Coastal security operations deploy 500+ interceptor boats, naval vessels with advanced weapons systems, and aircraft providing surveillance and rapid response Infrastructure security measures protect strategic ports, naval facilities, and critical communication installations from sabotage and terrorism Personnel training covers border patrolling techniques, threat recognition protocols, communication procedures, and emergency response Environmental monitoring identifies unusual activities including smuggling operations, infiltration attempts, and illegal maritime activities Technology provides early warning of aerial threats, vehicular movement detection, and precision identification of crossing points Intelligence sharing with international partners including Bangladesh, Myanmar, and Pakistan reduces transnational criminal activity Statistics tracking monitors penetration attempts, interdiction rates, and incident patterns informing continuous operational improvements
+Relevance: 21.2%
+---
+Document 12: Border Management and Coastal Security Operations Manual
+Content: Standard procedures for comprehensive management of 15,106 kilometers of land border and 7,517 kilometers of coastline Surveillance infrastructure encompasses 2,500+ surveillance cameras, comprehensive sensor networks, and real-time satellite imagery feeds Personnel deployment across all borders totals 500,000+ trained personnel providing continuous presence and rapid response capability Technology integration includes automated threat detection systems, unmanned drone patrols with extended flight endurance, and sensor fusion systems correlating multiple data sources for threat identification Coordination mechanisms link Border Security Force, Coast Guard, state police, and military units through unified command structures Cross-border incident protocols establish communication channels, rules for engagement, de-escalation procedures, and escalation pathways for different threat levels Coastal security operations deploy 500+ interceptor boats, naval vessels with advanced weapons systems, and aircraft providing surveillance and rapid response Infrastructure security measures protect strategic ports, naval facilities, and critical communication installations from sabotage and terrorism Personnel training covers border patrolling techniques, threat recognition protocols, communication procedures, and emergency response Environmental monitoring identifies unusual activities including smuggling operations, infiltration attempts, and illegal maritime activities Technology provides early warning of aerial threats, vehicular movement detection, and precision identification of crossing points Intelligence sharing with international partners including Bangladesh, Myanmar, and Pakistan reduces transnational criminal activity Statistics tracking monitors penetration attempts, interdiction rates, and incident patterns informing continuous operational improvements
+Relevance: 21.2%
+---
+Document 13: Veterans' Rehabilitation and Post-Service Support Program
+Content: The Veterans' Rehabilitation and Post-Service Support Program ensures dignified rehabilitation and reintegration of retired military personnel into civilian society Healthcare Services: - Free medical treatment for service-connected disabilities at defense hospitals - ECHS (Ex-Servicemen Contribution Health Scheme): Pan-India medical network coverage - Mental health support and PTSD counseling for combat trauma - Geriatric care centers for aging veterans and their dependents - Artificial limbs and prosthetics for disabled veterans Financial Support: - Disability pensions based on extent of disability (0-100%) - Pension reviews every 3 years with inflation adjustments - One-time rehabilitation grant for economically backward veterans - Interest-free loans for business startup and self-employment - Housing assistance and concessional housing schemes Employment Assistance: - Priority employment in civilian government and PSU jobs - Skill development courses in high-demand sectors - Self-employment training and business mentoring - Job placement assistance through employment fairs - Reservation in police forces and paramilitary organizations Education Support: - Scholarship programs for children of war casualties - Concessional admission to defense institutes and universities - Vocational training in engineering and trades - Adult literacy programs for less educated veterans Community Integration: - Veteran peer support groups and networking organizations - Recreational facilities and sports programs - Cultural programs and ceremonial recognition events - Grievance redressal mechanism for benefits disputes
+Relevance: 21.1%
+---
+Document 14: Unknown Document
+Content: 
+        The Veterans' Rehabilitation and Post-Service Support Program ensures dignified rehabilitation 
+        and reintegration of retired military personnel into civilian society.
+        Healthcare Services:
+        - Free medical treatment for service-connected disabilities at defense hospitals
+        - ECHS (Ex-Servicemen Contribution Health Scheme): Pan-India medical network coverage
+        - Mental health support and PTSD counseling for combat trauma
+        - Geriatric care centers for aging veterans and their dependents
+        - Artificial limbs and prosthetics for disabled veterans
+        Financial Support:
+        - Disability pensions based on extent of disability (0-100%)
+        - Pension reviews every 3 years with inflation adjustments
+        - One-time rehabilitation grant for economically backward veterans
+        - Interest-free loans for business startup and self-employment
+        - Housing assistance and concessional housing schemes
+        Employment Assistance:
+        - Priority employment in civilian government and PSU jobs
+        - Skill development courses in high-demand sectors
+        - Self-employment training and business mentoring
+        - Job placement assistance through employment fairs
+        - Reservation in police forces and paramilitary organizations
+        Education Support:
+        - Scholarship programs for children of war casualties
+        - Concessional admission to defense institutes and universities
+        - Vocational training in engineering and trades
+        - Adult literacy programs for less educated veterans
+        Community Integration:
+        - Veteran peer support groups and networking organizations
+        - Recreational facilities and sports programs
+        - Cultural programs and ceremonial recognition events
+        - Grievance redressal mechanism for benefits disputes
+Relevance: 21.1%
+---
+Document 15: Unknown Document
+Content: 
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        an</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>multi-model-synthesis</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>38.143235206604</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix ChromaDB telemetry and retry chunk generation
</commit_message>
<xml_diff>
--- a/data/generated_answers/rag_debug_logs.xlsx
+++ b/data/generated_answers/rag_debug_logs.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -4403,6 +4403,1530 @@
         <v>38.143235206604</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11T08:53:34.258181</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>what is the latest defence deal?</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document: Defence Procurement Policy 2023 - Strategic Framework
+Similarity: 0.5351043939590454
+Text:
+The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed 
+---------------------------------------
+Document: Defence Procurement Policy 2023 - Strategic Framework
+Similarity: 0.5141444206237793
+Text:
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include:
+        1. Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content.
+        2. Technology Transfer: Foreign vendors must commit to technology transfer agreements for strate
+---------------------------------------
+Document: Defence Budget Allocation 2023-24: Analysis and Distribution
+Similarity: 0.5127302408218384
+Text:
+The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime
+---------------------------------------
+Document: Defence Budget Allocation 2023-24: Analysis and Distribution
+Similarity: 0.5123133659362793
+Text:
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crore
+---------------------------------------
+Document: Cybersecurity Strategy for Defence Installations 2023
+Similarity: 0.4115431308746338
+Text:
+The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual p
+---------------------------------------
+Document: Cybersecurity Strategy for Defence Installations 2023
+Similarity: 0.4075409173965454
+Text:
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and cont
+---------------------------------------
+Document: Maritime Security Strategy for Indian Ocean Region
+Similarity: 0.3887385129928589
+Text:
+Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting
+---------------------------------------
+Document: Maritime Security Strategy for Indian Ocean Region
+Similarity: 0.3887385129928589
+Text:
+Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting
+---------------------------------------
+Document: Advanced Weaponry Systems: Development and Deployment
+Similarity: 0.377407431602478
+Text:
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km,
+---------------------------------------
+Document: Advanced Weaponry Systems: Development and Deployment
+Similarity: 0.37335795164108276
+Text:
+This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems </t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document 1: Defence Procurement Policy 2023 - Strategic Framework
+Content: The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems 4 Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts 5 Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, Contract Negotiation, and Implementation with quarterly reviews All decisions are documented for transparency Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements
+Relevance: 53.5%
+---
+Document 2: Unknown Document
+Content: 
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include:
+        1. Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content.
+        2. Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems.
+        3. FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems.
+        4. Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts.
+        5. Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years.
+        The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, 
+        Contract Negotiation, and Implementation with quarterly reviews. All decisions are documented for transparency.
+        Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development.
+        The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements.
+Relevance: 51.4%
+---
+Document 3: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 51.3%
+---
+Document 4: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 51.2%
+---
+Document 5: Cybersecurity Strategy for Defence Installations 2023
+Content: The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual property Defensive Measures: - Zero Trust Architecture: All access requires verification, no implicit trust - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256) - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens - Air-Gapped Networks: Critical systems isolated from internet connectivity - Continuous Monitoring: 24/7 intrusion detection and prevention systems Operational Protocols: - Defense Information Systems Agency (DISA) standards for network design - Regular penetration testing by authorized ethical hackers (quarterly) - Security incident response within 4 hours of detection - Personnel security clearances updated annually with background verification - Equipment procurement from certified vendors with security audits Incident Response: - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection - Forensics preserved for investigation and prosecution - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 41.2%
+---
+Document 6: Unknown Document
+Content: 
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and control systems
+        - Theft of defense technology and intellectual property
+        Defensive Measures:
+        - Zero Trust Architecture: All access requires verification, no implicit trust
+        - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256)
+        - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens
+        - Air-Gapped Networks: Critical systems isolated from internet connectivity
+        - Continuous Monitoring: 24/7 intrusion detection and prevention systems
+        Operational Protocols:
+        - Defense Information Systems Agency (DISA) standards for network design
+        - Regular penetration testing by authorized ethical hackers (quarterly)
+        - Security incident response within 4 hours of detection
+        - Personnel security clearances updated annually with background verification
+        - Equipment procurement from certified vendors with security audits
+        Incident Response:
+        - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection
+        - Forensics preserved for investigation and prosecution
+        - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 40.8%
+---
+Document 7: Maritime Security Strategy for Indian Ocean Region
+Content: Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting illegal activities The maritime security strategy recognizes India's critical economic dependence on sea lanes with 95% of external trade conducted through maritime routes Naval force modernization roadmap targets achieving 175 operational ships by 2035, with current fleet strength at 140 vessels Major construction programs include Project 15B destroyers (advanced sensor systems and guided missiles), Project 17A frigates (multi-role combat capability), Project 75I submarines (enhanced underwater warfare capability), and fleet support vessels Submarine capability expansion encompasses 24 total submarines including 6 nuclear-powered ballistic missile submarines (SSBNs) providing strategic deterrence and 4 nuclear-powered attack submarines (SSNs) for power projection Advanced surface platforms modernization includes carrier task forces with INS Vikrant-class aircraft carriers (indigenous development), naval aviation modernization with MiG-29K fighters and advanced helicopters, and integrated air defence systems providing layered protection Naval aviation expansion includes 100+ naval helicopters and 200+ maritime patrol aircraft distributed across operational commands Regional cooperation through the SAGAR (Security and Growth for All in the Region) initiative strengthens maritime security partnerships, while participation in Indian Ocean Rim Association enables coordinated responses to transnational maritime challenges Strategic chokepoints receive special attention with enhanced surveillance capabilities and rapid response forces, particularly Strait of Malacca, Strait of Hormuz, and other critical waterways Technology integration includes satellite-based ocean surveillance, real-time intelligence fusion, and automated threat detection systems Cyber maritime operations address emerging threats to port infrastructure and vessel navigation systems
+Relevance: 38.9%
+---
+Document 8: Maritime Security Strategy for Indian Ocean Region
+Content: Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting illegal activities The maritime security strategy recognizes India's critical economic dependence on sea lanes with 95% of external trade conducted through maritime routes Naval force modernization roadmap targets achieving 175 operational ships by 2035, with current fleet strength at 140 vessels Major construction programs include Project 15B destroyers (advanced sensor systems and guided missiles), Project 17A frigates (multi-role combat capability), Project 75I submarines (enhanced underwater warfare capability), and fleet support vessels Submarine capability expansion encompasses 24 total submarines including 6 nuclear-powered ballistic missile submarines (SSBNs) providing strategic deterrence and 4 nuclear-powered attack submarines (SSNs) for power projection Advanced surface platforms modernization includes carrier task forces with INS Vikrant-class aircraft carriers (indigenous development), naval aviation modernization with MiG-29K fighters and advanced helicopters, and integrated air defence systems providing layered protection Naval aviation expansion includes 100+ naval helicopters and 200+ maritime patrol aircraft distributed across operational commands Regional cooperation through the SAGAR (Security and Growth for All in the Region) initiative strengthens maritime security partnerships, while participation in Indian Ocean Rim Association enables coordinated responses to transnational maritime challenges Strategic chokepoints receive special attention with enhanced surveillance capabilities and rapid response forces, particularly Strait of Malacca, Strait of Hormuz, and other critical waterways Technology integration includes satellite-based ocean surveillance, real-time intelligence fusion, and automated threat detection systems Cyber maritime operations address emerging threats to port infrastructure and vessel navigation systems
+Relevance: 38.9%
+---
+Document 9: Unknown Document
+Content: 
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation
+        - PSLV/GSLV: Satellite launch systems with dual military applications
+        - Nirbhay: Subsonic cruise missile under development for extended range operations
+        Aircraft Systems:
+        - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems
+        - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades
+        - HAL Prachand: Indigenous light combat helicopter, 15 in operation
+        - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters
+        Naval Platforms:
+        - INS Vikramaditya: Carrier with integrated air defense and communications systems
+        - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+        - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles
+        - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection
+        Ground Systems:
+        - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems
+        - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation
+        - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 37.7%
+---
+Document 10: Advanced Weaponry Systems: Development and Deployment
+Content: This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems with dual military applications - Nirbhay: Subsonic cruise missile under development for extended range operations Aircraft Systems: - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades - HAL Prachand: Indigenous light combat helicopter, 15 in operation - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters Naval Platforms: - INS Vikramaditya: Carrier with integrated air defense and communications systems - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion) - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection Ground Systems: - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 37.3%
+---
+Document 11: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 35.3%
+---
+Document 12: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 35.3%
+---
+Document 13: Personnel Training and Professional Development in Armed Forces
+Content: The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - Basic Military Training Centers: 6-12 week initial training - Trade-specific Training: Pilots, engineers, medical, signals, etc - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs - Continuing Education: Annual refresher courses on latest tactics and technology Technology Training: - Pilot Training on Rafale, Tejas, and other aircraft - Submarine Crew Training: Advanced underwater warfare tactics - Cyber Warfare Training: Defense against digital threats - Artificial Intelligence Applications: Machine learning and autonomous systems - Unmanned Systems: Drone and robot operation and maintenance International Exchange: - Training exchanges with allied nations (USA, UK, France, Israel) - Joint exercises providing real-world training scenarios - Instructor attachments at foreign military academies - Participation in international military competitions Standards and Evaluation: - Rigorous evaluation standards ensuring combat readiness - Competency-based assessment of all critical skills - Regular audits of training effectiveness - Feedback loops for continuous improvement of curriculum
+Relevance: 32.0%
+---
+Document 14: Military Modernization Strategy: 2023-2035 Road Map
+Content: India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force capable of addressing emerging security challenges in the Indo-Pacific region Strategic Pillars: 1 Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development 2 Self-Reliance: 80% indigenous content in all new systems by 2030 3 Joint Operations: Enhanced interoperability between services through common C4I systems 4 Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection 5 Space Applications: Military satellites for surveillance, navigation, and communication Priority Areas: - Hypersonic Missiles: Mach 5+ cruise missiles under development - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication - AI Integration: Autonomous systems for surveillance and decision support - Quantum Computing: Encryption and cryptographic applications for secure communication - Artificial Intelligence: Machine learning for target identification and predictive maintenance Partnerships: - Technology partnerships with USA, France, Israel, Russia, and Japan - Co-development arrangements for systems like fighter jets and helicopters - Joint exercises and interoperability protocols with friendly nations Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics
+Relevance: 31.7%
+---
+Document 15: Unknown Document
+Content: 
+        India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force 
+        capable of addressing emerging security challenges in the Indo-Pacific region.
+        Strategic Pillars:
+        1. Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development
+        2. Self-Reliance: 80% indigenous content in all new systems by 2030
+        3. Joint Operations: Enhanced interoperability between services through common C4I systems
+        4. Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection
+        5. Space Applications: Military satellites for surveillance, navigation, and communication
+        Priority Areas:
+        - Hypersonic Missiles: Mach 5+ cruise missiles under development
+        - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication
+        - AI Integration: Autonomous systems for surveillance and decision support
+        - Quantum Computing: Encryption and cryptographic applications for secure communication
+        - Artificial Intelligence: Machine learning for target identification and predictive maintenance
+        Partnerships:
+        - Technology partnerships with USA, France, Israel, Russia, and Japan
+        - Co-development arrangements for systems like fighter jets and helicopters
+        - Joint exercises and interoperability protocols with friendly nations
+        Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics.
+Relevance: 31.6%
+</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a Defence Intelligence Assistant.
+DOCUMENTS:
+Document 1: Defence Procurement Policy 2023 - Strategic Framework
+Content: The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems 4 Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts 5 Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, Contract Negotiation, and Implementation with quarterly reviews All decisions are documented for transparency Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements
+Relevance: 53.5%
+---
+Document 2: Unknown Document
+Content: 
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include:
+        1. Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content.
+        2. Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems.
+        3. FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems.
+        4. Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts.
+        5. Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years.
+        The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, 
+        Contract Negotiation, and Implementation with quarterly reviews. All decisions are documented for transparency.
+        Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development.
+        The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements.
+Relevance: 51.4%
+---
+Document 3: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 51.3%
+---
+Document 4: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 51.2%
+---
+Document 5: Cybersecurity Strategy for Defence Installations 2023
+Content: The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual property Defensive Measures: - Zero Trust Architecture: All access requires verification, no implicit trust - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256) - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens - Air-Gapped Networks: Critical systems isolated from internet connectivity - Continuous Monitoring: 24/7 intrusion detection and prevention systems Operational Protocols: - Defense Information Systems Agency (DISA) standards for network design - Regular penetration testing by authorized ethical hackers (quarterly) - Security incident response within 4 hours of detection - Personnel security clearances updated annually with background verification - Equipment procurement from certified vendors with security audits Incident Response: - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection - Forensics preserved for investigation and prosecution - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 41.2%
+---
+Document 6: Unknown Document
+Content: 
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and control systems
+        - Theft of defense technology and intellectual property
+        Defensive Measures:
+        - Zero Trust Architecture: All access requires verification, no implicit trust
+        - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256)
+        - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens
+        - Air-Gapped Networks: Critical systems isolated from internet connectivity
+        - Continuous Monitoring: 24/7 intrusion detection and prevention systems
+        Operational Protocols:
+        - Defense Information Systems Agency (DISA) standards for network design
+        - Regular penetration testing by authorized ethical hackers (quarterly)
+        - Security incident response within 4 hours of detection
+        - Personnel security clearances updated annually with background verification
+        - Equipment procurement from certified vendors with security audits
+        Incident Response:
+        - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection
+        - Forensics preserved for investigation and prosecution
+        - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 40.8%
+---
+Document 7: Maritime Security Strategy for Indian Ocean Region
+Content: Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting illegal activities The maritime security strategy recognizes India's critical economic dependence on sea lanes with 95% of external trade conducted through maritime routes Naval force modernization roadmap targets achieving 175 operational ships by 2035, with current fleet strength at 140 vessels Major construction programs include Project 15B destroyers (advanced sensor systems and guided missiles), Project 17A frigates (multi-role combat capability), Project 75I submarines (enhanced underwater warfare capability), and fleet support vessels Submarine capability expansion encompasses 24 total submarines including 6 nuclear-powered ballistic missile submarines (SSBNs) providing strategic deterrence and 4 nuclear-powered attack submarines (SSNs) for power projection Advanced surface platforms modernization includes carrier task forces with INS Vikrant-class aircraft carriers (indigenous development), naval aviation modernization with MiG-29K fighters and advanced helicopters, and integrated air defence systems providing layered protection Naval aviation expansion includes 100+ naval helicopters and 200+ maritime patrol aircraft distributed across operational commands Regional cooperation through the SAGAR (Security and Growth for All in the Region) initiative strengthens maritime security partnerships, while participation in Indian Ocean Rim Association enables coordinated responses to transnational maritime challenges Strategic chokepoints receive special attention with enhanced surveillance capabilities and rapid response forces, particularly Strait of Malacca, Strait of Hormuz, and other critical waterways Technology integration includes satellite-based ocean surveillance, real-time intelligence fusion, and automated threat detection systems Cyber maritime operations address emerging threats to port infrastructure and vessel navigation systems
+Relevance: 38.9%
+---
+Document 8: Maritime Security Strategy for Indian Ocean Region
+Content: Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting illegal activities The maritime security strategy recognizes India's critical economic dependence on sea lanes with 95% of external trade conducted through maritime routes Naval force modernization roadmap targets achieving 175 operational ships by 2035, with current fleet strength at 140 vessels Major construction programs include Project 15B destroyers (advanced sensor systems and guided missiles), Project 17A frigates (multi-role combat capability), Project 75I submarines (enhanced underwater warfare capability), and fleet support vessels Submarine capability expansion encompasses 24 total submarines including 6 nuclear-powered ballistic missile submarines (SSBNs) providing strategic deterrence and 4 nuclear-powered attack submarines (SSNs) for power projection Advanced surface platforms modernization includes carrier task forces with INS Vikrant-class aircraft carriers (indigenous development), naval aviation modernization with MiG-29K fighters and advanced helicopters, and integrated air defence systems providing layered protection Naval aviation expansion includes 100+ naval helicopters and 200+ maritime patrol aircraft distributed across operational commands Regional cooperation through the SAGAR (Security and Growth for All in the Region) initiative strengthens maritime security partnerships, while participation in Indian Ocean Rim Association enables coordinated responses to transnational maritime challenges Strategic chokepoints receive special attention with enhanced surveillance capabilities and rapid response forces, particularly Strait of Malacca, Strait of Hormuz, and other critical waterways Technology integration includes satellite-based ocean surveillance, real-time intelligence fusion, and automated threat detection systems Cyber maritime operations address emerging threats to port infrastructure and vessel navigation systems
+Relevance: 38.9%
+---
+Document 9: Unknown Document
+Content: 
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation
+        - PSLV/GSLV: Satellite launch systems with dual military applications
+        - Nirbhay: Subsonic cruise missile under development for extended range operations
+        Aircraft Systems:
+        - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems
+        - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades
+        - HAL Prachand: Indigenous light combat helicopter, 15 in operation
+        - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters
+        Naval Platforms:
+        - INS Vikramaditya: Carrier with integrated air defense and communications systems
+        - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+        - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles
+        - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection
+        Ground Systems:
+        - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems
+        - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation
+        - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 37.7%
+---
+Document 10: Advanced Weaponry Systems: Development and Deployment
+Content: This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems with dual military applications - Nirbhay: Subsonic cruise missile under development for extended range operations Aircraft Systems: - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades - HAL Prachand: Indigenous light combat helicopter, 15 in operation - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters Naval Platforms: - INS Vikramaditya: Carrier with integrated air defense and communications systems - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion) - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection Ground Systems: - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 37.3%
+---
+Document 11: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 35.3%
+---
+Document 12: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 35.3%
+---
+Document 13: Personnel Training and Professional Development in Armed Forces
+Content: The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - Basic Military Training Centers: 6-12 week initial training - Trade-specific Training: Pilots, engineers, medical, signals, etc - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs - Continuing Education: Annual refresher courses on latest tactics and technology Technology Training: - Pilot Training on Rafale, Tejas, and other aircraft - Submarine Crew Training: Advanced underwater warfare tactics - Cyber Warfare Training: Defense against digital threats - Artificial Intelligence Applications: Machine learning and autonomous systems - Unmanned Systems: Drone and robot operation and maintenance International Exchange: - Training exchanges with allied nations (USA, UK, France, Israel) - Joint exercises providing real-world training scenarios - Instructor attachments at foreign military academies - Participation in international military competitions Standards and Evaluation: - Rigorous evaluation standards ensuring combat readiness - Competency-based assessment of all critical skills - Regular audits of training effectiveness - Feedback loops for continuous improvement of curriculum
+Relevance: 32.0%
+---
+Document 14: Military Modernization Strategy: 2023-2035 Road Map
+Content: India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force capable of addressing emerging security challenges in the Indo-Pacific region Strategic Pillars: 1 Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development 2 Self-Reliance: 80% indigenous content in all new systems by 2030 3 Joint Operations: Enhanced interoperability between services through common C4I systems 4 Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection 5 Space Applications: Military satellites for surveillance, navigation, and communication Priority Areas: - Hypersonic Missiles: Mach 5+ cruise missiles under development - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication - AI Integration: Autonomous systems for surveillance and decision support - Quantum Computing: Encryption and cryptographic applications for secure communication - Artificial Intelligence: Machine learning for target identification and predictive maintenance Partnerships: - Technology partnerships with USA, France, Israel, Russia, and Japan - Co-development arrangements for systems like fighter jets and helicopters - Joint exercises and interoperability protocols with friendly nations Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics
+Relevance: 31.7%
+---
+Document 15: Unknown Document
+Content: 
+        India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force 
+        capable of addressing emerging security challenges in the Indo-Pacific region.
+        Strategic Pillars:
+        1. Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development
+        2. Self-Reliance: 80% indigenous content in all new systems by 2030
+        3. Joint Operations: Enhanced interoperability between services through common C4I systems
+        4. Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection
+        5. Space Applications: Military satellites for surveillance, navigation, and communication
+        Priority Areas:
+        - Hypersonic Missiles: Mach 5+ cruise missiles under development
+        - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication
+        - AI Integration: Autonomous systems for surveillance and decision support
+        - Quantum Computing: Encryption and cryptographic applications for secure communication
+        - Artificial Intelligence: Machine learning for target identification and predictive maintenance
+        Partnerships:
+        - Technology partnerships with USA, France, Israel, Russia, and Japan
+        - Co-development arrangements for systems like fighter jets and helicopters
+        - Joint exercises and interoperability protocols with friendly nations
+        Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics.
+Relevance: 31.6%
+QUESTION:
+what is the latest defence deal?
+ANSWER:
+</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Based on the official documents, the latest defence deals and major projects funded in the 2023-24 budget include:
+*   **Project 75-I:** </t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the latest defence deals mentioned are:
+1. Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+2. Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+3. FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+4. Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+5. Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+These deals are mentioned in Document 3: Defence Budget Allocation 2023-24: Analysis and Distribution, and Document 4: Unknown Document, which appears to be a duplicate of Document 3.
+Additionally, Document 9: Unknown Document, and Document 10: Advanced Weaponry Systems: Development and Deployment, mention other defence deals, including:
+1. BrahMos Cruise Missile
+2. Akash-NG Air Defence System
+3. QRSAM
+4. PSLV/GSLV: Satellite launch systems
+5. Nirbhay: Subsonic cruise missile
+6. Rafale Fighter Jet: 36 aircraft on order from France
+7. Tejas Light Combat Aircraft: 83 aircraft approved
+8. HAL Prachand: Indigenous light combat helicopter
+9. INS Vikramaditya: Carrier with integrated air defense and communications systems
+10. Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+However, the context does not provide a specific date or timeline for these deals, so it is unclear which one is the latest.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Based on the retrieved documents:
+1. From 'Document' (confidence: 53.5%):
+   The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India In...
+2. From 'Defence Procurement Policy 2023 - Strategic Framework' (confidence: 51.4%):
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include...
+3. From 'Document' (confidence: 51.3%):
+   The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>EXECUTIVE SUMMARY:
+Question: what is the latest defence deal?
+Overview:
+This report synthesizes intelligence from three independent model analyses and a fallback summary. It highlights common findings, discrepancies, and operational implications.
+Combined Analysis:
+Gemini Analysis:
+Based on the official documents, the latest defence deals and major projects funded in the 2023-24 budget include:
+*   **Project 75-I:** 
+Groq Analysis:
+Based on the provided context, the latest defence deals mentioned are:
+1. Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+2. Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+3. FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+4. Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+5. Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+These deals are mentioned in Document 3: Defence Budget Allocation 2023-24: Analysis and Distribution, and Document 4: Unknown Document, which appears to be a duplicate of Document 3.
+Additionally, Document 9: Unknown Document, and Document 10: Advanced Weaponry Systems: Development and Deployment, mention other defence deals, including:
+1. BrahMos Cruise Missile
+2. Akash-NG Air Defence System
+3. QRSAM
+4. PSLV/GSLV: Satellite launch systems
+5. Nirbhay: Subsonic cruise missile
+6. Rafale Fighter Jet: 36 aircraft on order from France
+7. Tejas Light Combat Aircraft: 83 aircraft approved
+8. HAL Prachand: Indigenous light combat helicopter
+9. INS Vikramaditya: Carrier with integrated air defense and communications systems
+10. Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+However, the context does not provide a specific date or timeline for these deals, so it is unclear which one is the latest.
+Grok Analysis:
+No Grok output available.
+Fallback Analysis:
+Based on the retrieved documents:
+1. From 'Document' (confidence: 53.5%):
+   The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India In...
+2. From 'Defence Procurement Policy 2023 - Strategic Framework' (confidence: 51.4%):
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include...
+3. From 'Document' (confidence: 51.3%):
+   The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.
+Key Findings:
+- Gemini: Based on the official documents, the latest defence deals and major projects funded in the 2023-24 budget include:...
+- Groq: Based on the provided context, the latest defence deals mentioned are:...
+Detailed Analysis:
+Gemini Analysis:
+Based on the official documents, the latest defence deals and major projects funded in the 2023-24 budget include:
+*   **Project 75-I:** 
+Groq Analysis:
+Based on the provided context, the latest defence deals mentioned are:
+1. Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+2. Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+3. FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+4. Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+5. Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+These deals are mentioned in Document 3: Defence Budget Allocation 2023-24: Analysis and Distribution, and Document 4: Unknown Document, which appears to be a duplicate of Document 3.
+Additionally, Document 9: Unknown Document, and Document 10: Advanced Weaponry Systems: Development and Deployment, mention other defence deals, including:
+1. BrahMos Cruise Missile
+2. Akash-NG Air Defence System
+3. QRSAM
+4. PSLV/GSLV: Satellite launch systems
+5. Nirbhay: Subsonic cruise missile
+6. Rafale Fighter Jet: 36 aircraft on order from France
+7. Tejas Light Combat Aircraft: 83 aircraft approved
+8. HAL Prachand: Indigenous light combat helicopter
+9. INS Vikramaditya: Carrier with integrated air defense and communications systems
+10. Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+However, the context does not provide a specific date or timeline for these deals, so it is unclear which one is the latest.
+Grok Analysis:
+No Grok output available.
+Fallback Analysis:
+Based on the retrieved documents:
+1. From 'Document' (confidence: 53.5%):
+   The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India In...
+2. From 'Defence Procurement Policy 2023 - Strategic Framework' (confidence: 51.4%):
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include...
+3. From 'Document' (confidence: 51.3%):
+   The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.
+Retrieved Context and Sources:
+Document 1: Defence Procurement Policy 2023 - Strategic Framework
+Content: The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment and systems The policy emphasizes indigenous development, self-reliance, and technology transfer Key priorities include: 1 Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content 2 Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems 3 FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems 4 Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts 5 Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, Contract Negotiation, and Implementation with quarterly reviews All decisions are documented for transparency Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements
+Relevance: 53.5%
+---
+Document 2: Unknown Document
+Content: 
+        The Defence Procurement Policy 2023 establishes a comprehensive framework for acquisition of defence equipment 
+        and systems. The policy emphasizes indigenous development, self-reliance, and technology transfer. Key priorities include:
+        1. Make in India Initiative: Priority given to domestically manufactured defence systems with at least 50% indigenous content.
+        2. Technology Transfer: Foreign vendors must commit to technology transfer agreements for strategic systems.
+        3. FDI Enhancement: 100% FDI allowed in defence manufacturing with government approval for critical systems.
+        4. Transparent Procurement: e-bidding systems and real-time tracking of all defence contracts.
+        5. Gestation Support: Interest-free loans for MSMEs in defence manufacturing for first 5 years.
+        The procurement process involves: Request for Proposal (RFP), Technical Evaluation, Financial Bid Opening, 
+        Contract Negotiation, and Implementation with quarterly reviews. All decisions are documented for transparency.
+        Defence procurement now follows a 18-month timeline from RFP to contract award to accelerate capability development.
+        The policy applies to all three services: Army, Navy, and Air Force, with service-specific guidelines for their unique requirements.
+Relevance: 51.4%
+---
+Document 3: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 51.3%
+---
+Document 4: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 51.2%
+---
+Document 5: Cybersecurity Strategy for Defence Installations 2023
+Content: The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual property Defensive Measures: - Zero Trust Architecture: All access requires verification, no implicit trust - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256) - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens - Air-Gapped Networks: Critical systems isolated from internet connectivity - Continuous Monitoring: 24/7 intrusion detection and prevention systems Operational Protocols: - Defense Information Systems Agency (DISA) standards for network design - Regular penetration testing by authorized ethical hackers (quarterly) - Security incident response within 4 hours of detection - Personnel security clearances updated annually with background verification - Equipment procurement from certified vendors with security audits Incident Response: - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection - Forensics preserved for investigation and prosecution - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 41.2%
+---
+Document 6: Unknown Document
+Content: 
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and control systems
+        - Theft of defense technology and intellectual property
+        Defensive Measures:
+        - Zero Trust Architecture: All access requires verification, no implicit trust
+        - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256)
+        - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens
+        - Air-Gapped Networks: Critical systems isolated from internet connectivity
+        - Continuous Monitoring: 24/7 intrusion detection and prevention systems
+        Operational Protocols:
+        - Defense Information Systems Agency (DISA) standards for network design
+        - Regular penetration testing by authorized ethical hackers (quarterly)
+        - Security incident response within 4 hours of detection
+        - Personnel security clearances updated annually with background verification
+        - Equipment procurement from certified vendors with security audits
+        Incident Response:
+        - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection
+        - Forensics preserved for investigation and prosecution
+        - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 40.8%
+---
+Document 7: Maritime Security Strategy for Indian Ocean Region
+Content: Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting illegal activities The maritime security strategy recognizes India's critical economic dependence on sea lanes with 95% of external trade conducted through maritime routes Naval force modernization roadmap targets achieving 175 operational ships by 2035, with current fleet strength at 140 vessels Major construction programs include Project 15B destroyers (advanced sensor systems and guided missiles), Project 17A frigates (multi-role combat capability), Project 75I submarines (enhanced underwater warfare capability), and fleet support vessels Submarine capability expansion encompasses 24 total submarines including 6 nuclear-powered ballistic missile submarines (SSBNs) providing strategic deterrence and 4 nuclear-powered attack submarines (SSNs) for power projection Advanced surface platforms modernization includes carrier task forces with INS Vikrant-class aircraft carriers (indigenous development), naval aviation modernization with MiG-29K fighters and advanced helicopters, and integrated air defence systems providing layered protection Naval aviation expansion includes 100+ naval helicopters and 200+ maritime patrol aircraft distributed across operational commands Regional cooperation through the SAGAR (Security and Growth for All in the Region) initiative strengthens maritime security partnerships, while participation in Indian Ocean Rim Association enables coordinated responses to transnational maritime challenges Strategic chokepoints receive special attention with enhanced surveillance capabilities and rapid response forces, particularly Strait of Malacca, Strait of Hormuz, and other critical waterways Technology integration includes satellite-based ocean surveillance, real-time intelligence fusion, and automated threat detection systems Cyber maritime operations address emerging threats to port infrastructure and vessel navigation systems
+Relevance: 38.9%
+---
+Document 8: Maritime Security Strategy for Indian Ocean Region
+Content: Comprehensive maritime security framework encompassing 3 7 million square kilometers of maritime zone under Indian jurisdiction Strategic objectives for maritime operations include: freedom of navigation protection ensuring international shipping lanes remain open and secure, advanced anti-piracy operations leveraging satellite surveillance and naval patrol assets, counter-terrorism at sea targeting maritime militant groups, and environmental monitoring protecting marine ecosystems and detecting illegal activities The maritime security strategy recognizes India's critical economic dependence on sea lanes with 95% of external trade conducted through maritime routes Naval force modernization roadmap targets achieving 175 operational ships by 2035, with current fleet strength at 140 vessels Major construction programs include Project 15B destroyers (advanced sensor systems and guided missiles), Project 17A frigates (multi-role combat capability), Project 75I submarines (enhanced underwater warfare capability), and fleet support vessels Submarine capability expansion encompasses 24 total submarines including 6 nuclear-powered ballistic missile submarines (SSBNs) providing strategic deterrence and 4 nuclear-powered attack submarines (SSNs) for power projection Advanced surface platforms modernization includes carrier task forces with INS Vikrant-class aircraft carriers (indigenous development), naval aviation modernization with MiG-29K fighters and advanced helicopters, and integrated air defence systems providing layered protection Naval aviation expansion includes 100+ naval helicopters and 200+ maritime patrol aircraft distributed across operational commands Regional cooperation through the SAGAR (Security and Growth for All in the Region) initiative strengthens maritime security partnerships, while participation in Indian Ocean Rim Association enables coordinated responses to transnational maritime challenges Strategic chokepoints receive special attention with enhanced surveillance capabilities and rapid response forces, particularly Strait of Malacca, Strait of Hormuz, and other critical waterways Technology integration includes satellite-based ocean surveillance, real-time intelligence fusion, and automated threat detection systems Cyber maritime operations address emerging threats to port infrastructure and vessel navigation systems
+Relevance: 38.9%
+---
+Document 9: Unknown Document
+Content: 
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation
+        - PSLV/GSLV: Satellite launch systems with dual military applications
+        - Nirbhay: Subsonic cruise missile under development for extended range operations
+        Aircraft Systems:
+        - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems
+        - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades
+        - HAL Prachand: Indigenous light combat helicopter, 15 in operation
+        - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters
+        Naval Platforms:
+        - INS Vikramaditya: Carrier with integrated air defense and communications systems
+        - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+        - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles
+        - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection
+        Ground Systems:
+        - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems
+        - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation
+        - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 37.7%
+---
+Document 10: Advanced Weaponry Systems: Development and Deployment
+Content: This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems with dual military applications - Nirbhay: Subsonic cruise missile under development for extended range operations Aircraft Systems: - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades - HAL Prachand: Indigenous light combat helicopter, 15 in operation - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters Naval Platforms: - INS Vikramaditya: Carrier with integrated air defense and communications systems - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion) - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection Ground Systems: - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 37.3%
+---
+Document 11: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 35.3%
+---
+Document 12: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 35.3%
+---
+Document 13: Personnel Training and Professional Development in Armed Forces
+Content: The Armed Forces training and development program ensures that military personnel are equipped with cutting-edge knowledge and skills for modern warfare Officer Training Academies: - National Defence Academy (NDA): 4-year training for commission as officer - Officers Training Academy (OTA): 49-week training for graduate officers - Army Staff College: Senior officer strategy and leadership development - War Colleges: Highest level strategic and operational training Enlisted Personnel Training: - Basic Military Training Centers: 6-12 week initial training - Trade-specific Training: Pilots, engineers, medical, signals, etc - Leadership Schools: NCO (Non-Commissioned Officer) advancement programs - Continuing Education: Annual refresher courses on latest tactics and technology Technology Training: - Pilot Training on Rafale, Tejas, and other aircraft - Submarine Crew Training: Advanced underwater warfare tactics - Cyber Warfare Training: Defense against digital threats - Artificial Intelligence Applications: Machine learning and autonomous systems - Unmanned Systems: Drone and robot operation and maintenance International Exchange: - Training exchanges with allied nations (USA, UK, France, Israel) - Joint exercises providing real-world training scenarios - Instructor attachments at foreign military academies - Participation in international military competitions Standards and Evaluation: - Rigorous evaluation standards ensuring combat readiness - Competency-based assessment of all critical skills - Regular audits of training effectiveness - Feedback loops for continuous improvement of curriculum
+Relevance: 32.0%
+---
+Document 14: Military Modernization Strategy: 2023-2035 Road Map
+Content: India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force capable of addressing emerging security challenges in the Indo-Pacific region Strategic Pillars: 1 Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development 2 Self-Reliance: 80% indigenous content in all new systems by 2030 3 Joint Operations: Enhanced interoperability between services through common C4I systems 4 Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection 5 Space Applications: Military satellites for surveillance, navigation, and communication Priority Areas: - Hypersonic Missiles: Mach 5+ cruise missiles under development - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication - AI Integration: Autonomous systems for surveillance and decision support - Quantum Computing: Encryption and cryptographic applications for secure communication - Artificial Intelligence: Machine learning for target identification and predictive maintenance Partnerships: - Technology partnerships with USA, France, Israel, Russia, and Japan - Co-development arrangements for systems like fighter jets and helicopters - Joint exercises and interoperability protocols with friendly nations Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics
+Relevance: 31.7%
+---
+Document 15: Unknown Document
+Content: 
+        India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force 
+        capable of addressing emerging security challenges in the Indo-Pacific region.
+        Strategic Pillars:
+        1. Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development
+        2. Self-Reliance: 80% indigenous content in all new systems by 2030
+        3. Joint Operations: Enhanced interoperability between services through common C4I systems
+        4. Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection
+        5. Space Applications: Military satellites for surveillance, navigation, and communication
+        Priority Areas:
+        - Hypersonic Missiles: Mach 5+ cruise missiles under development
+        - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication
+        - AI Integration: Autonomous systems for surveillance and decision support
+        - Quantum Computing: Encryption and cryptographic applications for secure communication
+        - Artificial Intelligence: Machine learning for target identification and predictive maintenance
+        Partnerships:
+        - Technology partnerships with USA, France, Israel, Russia, and Japan
+        - Co-development arrangements for systems like fighter jets and helicopters
+        - Joint exercises and interoperability protocols with friendly nations
+        Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics.
+Relevance: 31.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>multi-model-synthesis</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>44.46547436714172</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11T11:45:11.704926</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>tell me about latest news related to drdo</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document: Defence Research and Development: Innovation in Military Technology
+Similarity: 0.35793066024780273
+Text:
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Development Establishment (ADE): Aircraft and missile design
+        - Defence Electronics Research Laboratory (DERL): Electronics and communications
+        - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles
+        - Naval Scien
+---------------------------------------
+Document: Defence Research and Development: Innovation in Military Technology
+Similarity: 0.34512364864349365
+Text:
+The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile design - Defence Electronics Research Laboratory (DERL): Electronics and communications - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles - Naval Science and Technological Laboratory (NSTL): Submarine and ship technolog
+---------------------------------------
+Document: Cybersecurity Strategy for Defence Installations 2023
+Similarity: 0.13202685117721558
+Text:
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and cont
+---------------------------------------
+Document: Defence Budget Allocation 2023-24: Analysis and Distribution
+Similarity: 0.13178694248199463
+Text:
+The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime
+---------------------------------------
+Document: Advanced Weaponry Systems: Development and Deployment
+Similarity: 0.1303718090057373
+Text:
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km,
+---------------------------------------
+Document: Cybersecurity Strategy for Defence Installations 2023
+Similarity: 0.12923157215118408
+Text:
+The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual p
+---------------------------------------
+Document: Defence Budget Allocation 2023-24: Analysis and Distribution
+Similarity: 0.12755411863327026
+Text:
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crore
+---------------------------------------
+Document: Advanced Weaponry Systems: Development and Deployment
+Similarity: 0.12363278865814209
+Text:
+This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems 
+---------------------------------------
+Document: Indo-Pacific Security and Regional Defence Cooperation
+Similarity: 0.1215786337852478
+Text:
+        India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast 
+        area with significant maritime trade routes and strategic importance.
+        Regional Challenges:
+        - Maritime disputes in South China Sea and Indian Ocean
+        - Terrorism and extremism affecting coastal security
+        - Piracy and armed robbery in key shipping lanes
+        - Unregulated arms trafficking and human trafficking
+        - Climat
+---------------------------------------
+Document: Indo-Pacific Security and Regional Defence Cooperation
+Similarity: 0.1207539439201355
+Text:
+India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast area with significant maritime trade routes and strategic importance Regional Challenges: - Maritime disputes in South China Sea and Indian Ocean - Terrorism and extremism affecting coastal security - Piracy and armed robbery in key shipping lanes - Unregulated arms trafficking and human trafficking - Climate change impacts on island nations and maritime zones Defence Partnerships: </t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Document 1: Unknown Document
+Content: 
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Development Establishment (ADE): Aircraft and missile design
+        - Defence Electronics Research Laboratory (DERL): Electronics and communications
+        - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles
+        - Naval Science and Technological Laboratory (NSTL): Submarine and ship technology
+        - Centre for Airborne Systems (CARS): Avionics and mission systems
+        Major Projects:
+        - FRCN: Fifth Generation Combat Aircraft (stealth, AI-enabled)
+        - ASTRA Missile: Air-to-air missile with indigenous seekers and propulsion
+        - Lakshya Target: Unmanned aerial vehicle for training and reconnaissance
+        - Tactical Ballistic Missile (TBM): Short-range precision strike system
+        Advanced Technologies:
+        - Directed Energy Weapons: High-power laser and microwave systems
+        - Quantum Radar: Detection system using quantum entanglement properties
+        - Additive Manufacturing: 3D printing for complex defense components
+        - Artificial Intelligence: Machine learning for autonomous systems
+        - Biotechnology: Biological sensors and health monitoring systems
+        Collaboration:
+        - Industry partnerships with private sector for rapid development
+        - Academic collaborations with universities for research
+        - International partnerships with friendly nations for technology exchange
+        - Startup ecosystem fostering innovation in defense tech startups
+        Patents and Intellectual Property:
+        - Over 400 patents filed in last 5 years in critical defense technologies
+        - Technology transfer to private industry for commercial applications
+        - Open innovation platforms for crowd-sourced problem solving
+Relevance: 35.8%
+---
+Document 2: Defence Research and Development: Innovation in Military Technology
+Content: The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile design - Defence Electronics Research Laboratory (DERL): Electronics and communications - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles - Naval Science and Technological Laboratory (NSTL): Submarine and ship technology - Centre for Airborne Systems (CARS): Avionics and mission systems Major Projects: - FRCN: Fifth Generation Combat Aircraft (stealth, AI-enabled) - ASTRA Missile: Air-to-air missile with indigenous seekers and propulsion - Lakshya Target: Unmanned aerial vehicle for training and reconnaissance - Tactical Ballistic Missile (TBM): Short-range precision strike system Advanced Technologies: - Directed Energy Weapons: High-power laser and microwave systems - Quantum Radar: Detection system using quantum entanglement properties - Additive Manufacturing: 3D printing for complex defense components - Artificial Intelligence: Machine learning for autonomous systems - Biotechnology: Biological sensors and health monitoring systems Collaboration: - Industry partnerships with private sector for rapid development - Academic collaborations with universities for research - International partnerships with friendly nations for technology exchange - Startup ecosystem fostering innovation in defense tech startups Patents and Intellectual Property: - Over 400 patents filed in last 5 years in critical defense technologies - Technology transfer to private industry for commercial applications - Open innovation platforms for crowd-sourced problem solving
+Relevance: 34.5%
+---
+Document 3: Unknown Document
+Content: 
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and control systems
+        - Theft of defense technology and intellectual property
+        Defensive Measures:
+        - Zero Trust Architecture: All access requires verification, no implicit trust
+        - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256)
+        - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens
+        - Air-Gapped Networks: Critical systems isolated from internet connectivity
+        - Continuous Monitoring: 24/7 intrusion detection and prevention systems
+        Operational Protocols:
+        - Defense Information Systems Agency (DISA) standards for network design
+        - Regular penetration testing by authorized ethical hackers (quarterly)
+        - Security incident response within 4 hours of detection
+        - Personnel security clearances updated annually with background verification
+        - Equipment procurement from certified vendors with security audits
+        Incident Response:
+        - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection
+        - Forensics preserved for investigation and prosecution
+        - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 13.2%
+---
+Document 4: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 13.2%
+---
+Document 5: Unknown Document
+Content: 
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation
+        - PSLV/GSLV: Satellite launch systems with dual military applications
+        - Nirbhay: Subsonic cruise missile under development for extended range operations
+        Aircraft Systems:
+        - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems
+        - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades
+        - HAL Prachand: Indigenous light combat helicopter, 15 in operation
+        - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters
+        Naval Platforms:
+        - INS Vikramaditya: Carrier with integrated air defense and communications systems
+        - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+        - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles
+        - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection
+        Ground Systems:
+        - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems
+        - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation
+        - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 13.0%
+---
+Document 6: Cybersecurity Strategy for Defence Installations 2023
+Content: The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual property Defensive Measures: - Zero Trust Architecture: All access requires verification, no implicit trust - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256) - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens - Air-Gapped Networks: Critical systems isolated from internet connectivity - Continuous Monitoring: 24/7 intrusion detection and prevention systems Operational Protocols: - Defense Information Systems Agency (DISA) standards for network design - Regular penetration testing by authorized ethical hackers (quarterly) - Security incident response within 4 hours of detection - Personnel security clearances updated annually with background verification - Equipment procurement from certified vendors with security audits Incident Response: - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection - Forensics preserved for investigation and prosecution - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 12.9%
+---
+Document 7: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 12.8%
+---
+Document 8: Advanced Weaponry Systems: Development and Deployment
+Content: This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems with dual military applications - Nirbhay: Subsonic cruise missile under development for extended range operations Aircraft Systems: - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades - HAL Prachand: Indigenous light combat helicopter, 15 in operation - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters Naval Platforms: - INS Vikramaditya: Carrier with integrated air defense and communications systems - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion) - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection Ground Systems: - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 12.4%
+---
+Document 9: Unknown Document
+Content: 
+        India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast 
+        area with significant maritime trade routes and strategic importance.
+        Regional Challenges:
+        - Maritime disputes in South China Sea and Indian Ocean
+        - Terrorism and extremism affecting coastal security
+        - Piracy and armed robbery in key shipping lanes
+        - Unregulated arms trafficking and human trafficking
+        - Climate change impacts on island nations and maritime zones
+        Defence Partnerships:
+        - Quad Alliance: USA, Japan, Australia, India cooperation for peace and stability
+        - BIMSTEC: Bay of Bengal Initiative for regional security cooperation
+        - ASEAN Engagement: Strategic dialogue and military cooperation exercises
+        - Indian Ocean Rim Association: Coordination for maritime security
+        Operational Activities:
+        - Regular naval exercises: Malabar (USA, Japan, India), MILAN (regional navies)
+        - Joint air exercises with friendly nations to build interoperability
+        - Anti-piracy operations in Gulf of Aden and Indian Ocean
+        - Disaster relief and humanitarian assistance missions
+        Technology and Intelligence Sharing:
+        - Real-time information sharing on maritime threats and piracy
+        - Joint surveillance operations in critical sea lanes
+        - Coordinated response to emerging security threats
+        - Exchange of intelligence on terrorism and extremism funding
+        Future Strategy:
+        - Strengthening missile defense capabilities for regional credibility
+        - Expanding naval presence with additional carrier battle groups
+        - Building indigenous space-based surveillance and early warning systems
+        - Enhanced cyber defense for critical maritime and port infrastructure
+Relevance: 12.2%
+---
+Document 10: Indo-Pacific Security and Regional Defence Cooperation
+Content: India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast area with significant maritime trade routes and strategic importance Regional Challenges: - Maritime disputes in South China Sea and Indian Ocean - Terrorism and extremism affecting coastal security - Piracy and armed robbery in key shipping lanes - Unregulated arms trafficking and human trafficking - Climate change impacts on island nations and maritime zones Defence Partnerships: - Quad Alliance: USA, Japan, Australia, India cooperation for peace and stability - BIMSTEC: Bay of Bengal Initiative for regional security cooperation - ASEAN Engagement: Strategic dialogue and military cooperation exercises - Indian Ocean Rim Association: Coordination for maritime security Operational Activities: - Regular naval exercises: Malabar (USA, Japan, India), MILAN (regional navies) - Joint air exercises with friendly nations to build interoperability - Anti-piracy operations in Gulf of Aden and Indian Ocean - Disaster relief and humanitarian assistance missions Technology and Intelligence Sharing: - Real-time information sharing on maritime threats and piracy - Joint surveillance operations in critical sea lanes - Coordinated response to emerging security threats - Exchange of intelligence on terrorism and extremism funding Future Strategy: - Strengthening missile defense capabilities for regional credibility - Expanding naval presence with additional carrier battle groups - Building indigenous space-based surveillance and early warning systems - Enhanced cyber defense for critical maritime and port infrastructure
+Relevance: 12.1%
+---
+Document 11: Military Modernization Strategy: 2023-2035 Road Map
+Content: India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force capable of addressing emerging security challenges in the Indo-Pacific region Strategic Pillars: 1 Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development 2 Self-Reliance: 80% indigenous content in all new systems by 2030 3 Joint Operations: Enhanced interoperability between services through common C4I systems 4 Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection 5 Space Applications: Military satellites for surveillance, navigation, and communication Priority Areas: - Hypersonic Missiles: Mach 5+ cruise missiles under development - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication - AI Integration: Autonomous systems for surveillance and decision support - Quantum Computing: Encryption and cryptographic applications for secure communication - Artificial Intelligence: Machine learning for target identification and predictive maintenance Partnerships: - Technology partnerships with USA, France, Israel, Russia, and Japan - Co-development arrangements for systems like fighter jets and helicopters - Joint exercises and interoperability protocols with friendly nations Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics
+Relevance: 11.4%
+---
+Document 12: Joint Theatre Command Implementation Roadmap
+Content: Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Theatre (Indian Ocean), Cyber Theatre (digital warfare operations), Space Theatre (satellite operations and space defence) Expected efficiency gains from unification: 15-20% reduction in administrative overhead and redundant support structures, faster decision-making cycles through simplified command chains, improved inter-service coordination eliminating compartmentalization, and better resource optimization Transition timeline structured in three phases: Phase 1 (2024-25) establishes new command structures with compatible organizational frameworks; Phase 2 (2025-26) implements resource consolidation with integrated logistics and personnel management; Phase 3 (2026-27) achieves full operationalization with theatre-level integrated exercises demonstrating seamless inter-service coordination Risk mitigation strategies address potential institutional disruption through: smooth transition protocols minimizing operational gaps, comprehensive training programs for officers and support staff adapting to new command structures, maintenance of continuity during transition period, and retention mechanisms for experienced personnel Technology integration includes unified command and control systems, real-time data sharing across services, and AI-based decision support systems providing situational assessment and recommendation synthesis Performance metrics for successful theatre command implementation include reduced decision-making timelines, improved operational effectiveness metrics, enhanced inter-service coordination demonstrated through joint exercises, and cost optimization targets The transformation represents major institutional change requiring sustained commitment from military leadership, government support, and international partnerships with allied nations having similar structures
+Relevance: 11.0%
+---
+Document 13: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 10.9%
+---
+Document 14: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 10.9%
+---
+Document 15: Unknown Document
+Content: 
+        India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force 
+        capable of addressing emerging security challenges in the Indo-Pacific region.
+        Strategic Pillars:
+        1. Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development
+        2. Self-Reliance: 80% indigenous content in all new systems by 2030
+        3. Joint Operations: Enhanced interoperability between services through common C4I systems
+        4. Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection
+        5. Space Applications: Military satellites for surveillance, navigation, and communication
+        Priority Areas:
+        - Hypersonic Missiles: Mach 5+ cruise missiles under development
+        - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication
+        - AI Integration: Autonomous systems for surveillance and decision support
+        - Quantum Computing: Encryption and cryptographic applications for secure communication
+        - Artificial Intelligence: Machine learning for target identification and predictive maintenance
+        Partnerships:
+        - Technology partnerships with USA, France, Israel, Russia, and Japan
+        - Co-development arrangements for systems like fighter jets and helicopters
+        - Joint exercises and interoperability protocols with friendly nations
+        Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics.
+Relevance: 10.8%
+</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">You are a Defence Intelligence Assistant.
+DOCUMENTS:
+Document 1: Unknown Document
+Content: 
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Development Establishment (ADE): Aircraft and missile design
+        - Defence Electronics Research Laboratory (DERL): Electronics and communications
+        - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles
+        - Naval Science and Technological Laboratory (NSTL): Submarine and ship technology
+        - Centre for Airborne Systems (CARS): Avionics and mission systems
+        Major Projects:
+        - FRCN: Fifth Generation Combat Aircraft (stealth, AI-enabled)
+        - ASTRA Missile: Air-to-air missile with indigenous seekers and propulsion
+        - Lakshya Target: Unmanned aerial vehicle for training and reconnaissance
+        - Tactical Ballistic Missile (TBM): Short-range precision strike system
+        Advanced Technologies:
+        - Directed Energy Weapons: High-power laser and microwave systems
+        - Quantum Radar: Detection system using quantum entanglement properties
+        - Additive Manufacturing: 3D printing for complex defense components
+        - Artificial Intelligence: Machine learning for autonomous systems
+        - Biotechnology: Biological sensors and health monitoring systems
+        Collaboration:
+        - Industry partnerships with private sector for rapid development
+        - Academic collaborations with universities for research
+        - International partnerships with friendly nations for technology exchange
+        - Startup ecosystem fostering innovation in defense tech startups
+        Patents and Intellectual Property:
+        - Over 400 patents filed in last 5 years in critical defense technologies
+        - Technology transfer to private industry for commercial applications
+        - Open innovation platforms for crowd-sourced problem solving
+Relevance: 35.8%
+---
+Document 2: Defence Research and Development: Innovation in Military Technology
+Content: The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile design - Defence Electronics Research Laboratory (DERL): Electronics and communications - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles - Naval Science and Technological Laboratory (NSTL): Submarine and ship technology - Centre for Airborne Systems (CARS): Avionics and mission systems Major Projects: - FRCN: Fifth Generation Combat Aircraft (stealth, AI-enabled) - ASTRA Missile: Air-to-air missile with indigenous seekers and propulsion - Lakshya Target: Unmanned aerial vehicle for training and reconnaissance - Tactical Ballistic Missile (TBM): Short-range precision strike system Advanced Technologies: - Directed Energy Weapons: High-power laser and microwave systems - Quantum Radar: Detection system using quantum entanglement properties - Additive Manufacturing: 3D printing for complex defense components - Artificial Intelligence: Machine learning for autonomous systems - Biotechnology: Biological sensors and health monitoring systems Collaboration: - Industry partnerships with private sector for rapid development - Academic collaborations with universities for research - International partnerships with friendly nations for technology exchange - Startup ecosystem fostering innovation in defense tech startups Patents and Intellectual Property: - Over 400 patents filed in last 5 years in critical defense technologies - Technology transfer to private industry for commercial applications - Open innovation platforms for crowd-sourced problem solving
+Relevance: 34.5%
+---
+Document 3: Unknown Document
+Content: 
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and control systems
+        - Theft of defense technology and intellectual property
+        Defensive Measures:
+        - Zero Trust Architecture: All access requires verification, no implicit trust
+        - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256)
+        - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens
+        - Air-Gapped Networks: Critical systems isolated from internet connectivity
+        - Continuous Monitoring: 24/7 intrusion detection and prevention systems
+        Operational Protocols:
+        - Defense Information Systems Agency (DISA) standards for network design
+        - Regular penetration testing by authorized ethical hackers (quarterly)
+        - Security incident response within 4 hours of detection
+        - Personnel security clearances updated annually with background verification
+        - Equipment procurement from certified vendors with security audits
+        Incident Response:
+        - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection
+        - Forensics preserved for investigation and prosecution
+        - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 13.2%
+---
+Document 4: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 13.2%
+---
+Document 5: Unknown Document
+Content: 
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation
+        - PSLV/GSLV: Satellite launch systems with dual military applications
+        - Nirbhay: Subsonic cruise missile under development for extended range operations
+        Aircraft Systems:
+        - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems
+        - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades
+        - HAL Prachand: Indigenous light combat helicopter, 15 in operation
+        - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters
+        Naval Platforms:
+        - INS Vikramaditya: Carrier with integrated air defense and communications systems
+        - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+        - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles
+        - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection
+        Ground Systems:
+        - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems
+        - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation
+        - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 13.0%
+---
+Document 6: Cybersecurity Strategy for Defence Installations 2023
+Content: The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual property Defensive Measures: - Zero Trust Architecture: All access requires verification, no implicit trust - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256) - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens - Air-Gapped Networks: Critical systems isolated from internet connectivity - Continuous Monitoring: 24/7 intrusion detection and prevention systems Operational Protocols: - Defense Information Systems Agency (DISA) standards for network design - Regular penetration testing by authorized ethical hackers (quarterly) - Security incident response within 4 hours of detection - Personnel security clearances updated annually with background verification - Equipment procurement from certified vendors with security audits Incident Response: - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection - Forensics preserved for investigation and prosecution - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 12.9%
+---
+Document 7: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 12.8%
+---
+Document 8: Advanced Weaponry Systems: Development and Deployment
+Content: This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems with dual military applications - Nirbhay: Subsonic cruise missile under development for extended range operations Aircraft Systems: - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades - HAL Prachand: Indigenous light combat helicopter, 15 in operation - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters Naval Platforms: - INS Vikramaditya: Carrier with integrated air defense and communications systems - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion) - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection Ground Systems: - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 12.4%
+---
+Document 9: Unknown Document
+Content: 
+        India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast 
+        area with significant maritime trade routes and strategic importance.
+        Regional Challenges:
+        - Maritime disputes in South China Sea and Indian Ocean
+        - Terrorism and extremism affecting coastal security
+        - Piracy and armed robbery in key shipping lanes
+        - Unregulated arms trafficking and human trafficking
+        - Climate change impacts on island nations and maritime zones
+        Defence Partnerships:
+        - Quad Alliance: USA, Japan, Australia, India cooperation for peace and stability
+        - BIMSTEC: Bay of Bengal Initiative for regional security cooperation
+        - ASEAN Engagement: Strategic dialogue and military cooperation exercises
+        - Indian Ocean Rim Association: Coordination for maritime security
+        Operational Activities:
+        - Regular naval exercises: Malabar (USA, Japan, India), MILAN (regional navies)
+        - Joint air exercises with friendly nations to build interoperability
+        - Anti-piracy operations in Gulf of Aden and Indian Ocean
+        - Disaster relief and humanitarian assistance missions
+        Technology and Intelligence Sharing:
+        - Real-time information sharing on maritime threats and piracy
+        - Joint surveillance operations in critical sea lanes
+        - Coordinated response to emerging security threats
+        - Exchange of intelligence on terrorism and extremism funding
+        Future Strategy:
+        - Strengthening missile defense capabilities for regional credibility
+        - Expanding naval presence with additional carrier battle groups
+        - Building indigenous space-based surveillance and early warning systems
+        - Enhanced cyber defense for critical maritime and port infrastructure
+Relevance: 12.2%
+---
+Document 10: Indo-Pacific Security and Regional Defence Cooperation
+Content: India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast area with significant maritime trade routes and strategic importance Regional Challenges: - Maritime disputes in South China Sea and Indian Ocean - Terrorism and extremism affecting coastal security - Piracy and armed robbery in key shipping lanes - Unregulated arms trafficking and human trafficking - Climate change impacts on island nations and maritime zones Defence Partnerships: - Quad Alliance: USA, Japan, Australia, India cooperation for peace and stability - BIMSTEC: Bay of Bengal Initiative for regional security cooperation - ASEAN Engagement: Strategic dialogue and military cooperation exercises - Indian Ocean Rim Association: Coordination for maritime security Operational Activities: - Regular naval exercises: Malabar (USA, Japan, India), MILAN (regional navies) - Joint air exercises with friendly nations to build interoperability - Anti-piracy operations in Gulf of Aden and Indian Ocean - Disaster relief and humanitarian assistance missions Technology and Intelligence Sharing: - Real-time information sharing on maritime threats and piracy - Joint surveillance operations in critical sea lanes - Coordinated response to emerging security threats - Exchange of intelligence on terrorism and extremism funding Future Strategy: - Strengthening missile defense capabilities for regional credibility - Expanding naval presence with additional carrier battle groups - Building indigenous space-based surveillance and early warning systems - Enhanced cyber defense for critical maritime and port infrastructure
+Relevance: 12.1%
+---
+Document 11: Military Modernization Strategy: 2023-2035 Road Map
+Content: India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force capable of addressing emerging security challenges in the Indo-Pacific region Strategic Pillars: 1 Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development 2 Self-Reliance: 80% indigenous content in all new systems by 2030 3 Joint Operations: Enhanced interoperability between services through common C4I systems 4 Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection 5 Space Applications: Military satellites for surveillance, navigation, and communication Priority Areas: - Hypersonic Missiles: Mach 5+ cruise missiles under development - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication - AI Integration: Autonomous systems for surveillance and decision support - Quantum Computing: Encryption and cryptographic applications for secure communication - Artificial Intelligence: Machine learning for target identification and predictive maintenance Partnerships: - Technology partnerships with USA, France, Israel, Russia, and Japan - Co-development arrangements for systems like fighter jets and helicopters - Joint exercises and interoperability protocols with friendly nations Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics
+Relevance: 11.4%
+---
+Document 12: Joint Theatre Command Implementation Roadmap
+Content: Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Theatre (Indian Ocean), Cyber Theatre (digital warfare operations), Space Theatre (satellite operations and space defence) Expected efficiency gains from unification: 15-20% reduction in administrative overhead and redundant support structures, faster decision-making cycles through simplified command chains, improved inter-service coordination eliminating compartmentalization, and better resource optimization Transition timeline structured in three phases: Phase 1 (2024-25) establishes new command structures with compatible organizational frameworks; Phase 2 (2025-26) implements resource consolidation with integrated logistics and personnel management; Phase 3 (2026-27) achieves full operationalization with theatre-level integrated exercises demonstrating seamless inter-service coordination Risk mitigation strategies address potential institutional disruption through: smooth transition protocols minimizing operational gaps, comprehensive training programs for officers and support staff adapting to new command structures, maintenance of continuity during transition period, and retention mechanisms for experienced personnel Technology integration includes unified command and control systems, real-time data sharing across services, and AI-based decision support systems providing situational assessment and recommendation synthesis Performance metrics for successful theatre command implementation include reduced decision-making timelines, improved operational effectiveness metrics, enhanced inter-service coordination demonstrated through joint exercises, and cost optimization targets The transformation represents major institutional change requiring sustained commitment from military leadership, government support, and international partnerships with allied nations having similar structures
+Relevance: 11.0%
+---
+Document 13: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 10.9%
+---
+Document 14: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 10.9%
+---
+Document 15: Unknown Document
+Content: 
+        India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force 
+        capable of addressing emerging security challenges in the Indo-Pacific region.
+        Strategic Pillars:
+        1. Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development
+        2. Self-Reliance: 80% indigenous content in all new systems by 2030
+        3. Joint Operations: Enhanced interoperability between services through common C4I systems
+        4. Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection
+        5. Space Applications: Military satellites for surveillance, navigation, and communication
+        Priority Areas:
+        - Hypersonic Missiles: Mach 5+ cruise missiles under development
+        - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication
+        - AI Integration: Autonomous systems for surveillance and decision support
+        - Quantum Computing: Encryption and cryptographic applications for secure communication
+        - Artificial Intelligence: Machine learning for target identification and predictive maintenance
+        Partnerships:
+        - Technology partnerships with USA, France, Israel, Russia, and Japan
+        - Co-development arrangements for systems like fighter jets and helicopters
+        - Joint exercises and interoperability protocols with friendly nations
+        Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics.
+Relevance: 10.8%
+QUESTION:
+tell me about latest news related to drdo
+ANSWER:
+</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Based on the provided documents, the Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution focused on achieving technological self-reliance and innovation in defence systems.
+Here's an overview of DRDO's activities and focus areas:
+**Research Laboratories:**
+*   **Aeronautical Development Establishment (ADE):** Specializes in aircraft and missile design.
+*   **Defence Electronics Research Laboratory (DERL):** Focuses on electronics and communications.
+*   **Mechanical Engineering Research Laboratory (MERL):** Works on ground systems and vehicles.
+*   **Naval Science and Technological Laboratory (NSTL):** Dedicated to submarine and ship technology.
+*   **Centre for Airborne Systems (CARS):** Develops avionics and mission systems.
+**Major Projects:**
+*   **FRCN:** A Fifth Generation Combat Aircraft project, incorporating stealth and AI-enabled capabilities.
+*   **ASTRA Missile:** An air-to-air missile featuring indigenous seekers and propulsion.
+*   **Lakshya Target:** An unmanned aerial vehicle used for training and reconnaissance.
+*   **Tactical Ballistic Missile (TBM):** A short-range precision strike system.
+**Advanced Technologies under Development:**
+*   **Directed Energy Weapons:** High-power laser and microwave systems.
+*   **Quantum Radar:** Detection systems utilizing quantum entanglement properties.
+*   **Additive</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the latest news related to DRDO (Defence Research and Development Organisation) includes:
+1. **Advanced Technologies**: DRDO is working on various advanced technologies such as Directed Energy Weapons, Quantum Radar, Additive Manufacturing, Artificial Intelligence, and Biotechnology.
+2. **Major Projects**: DRDO is involved in several major projects, including the development of the Fifth Generation Combat Aircraft (FRCN), ASTRA Missile, Lakshya Target, and Tactical Ballistic Missile (TBM).
+3. **Collaboration**: DRDO is collaborating with industry partners, academic institutions, and international organizations to accelerate the development of defence technologies.
+4. **Patents and Intellectual Property**: DRDO has filed over 400 patents in the last 5 years in critical defence technologies and is working on technology transfer to private industry for commercial applications.
+5. **Research Laboratories**: DRDO has several research laboratories, including the Aeronautical Development Establishment (ADE), Defence Electronics Research Laboratory (DERL), Mechanical Engineering Research Laboratory (MERL), Naval Science and Technological Laboratory (NSTL), and Centre for Airborne Systems (CARS).
+However, it's worth noting that the provided context does not include real-time news or updates. The information is based on the documents provided, which may not reflect the latest developments or news related to DRDO.
+If you're looking for the latest news on DRDO, I recommend checking reputable news sources or the official DRDO website for the most up-to-date information.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Based on the retrieved documents:
+1. From 'Defence Research and Development: Innovation in Military Technology' (confidence: 35.8%):
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Developmen...
+2. From 'Document' (confidence: 34.5%):
+   The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile ...
+3. From 'Cybersecurity Strategy for Defence Installations 2023' (confidence: 13.2%):
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>EXECUTIVE SUMMARY:
+Question: tell me about latest news related to drdo
+Overview:
+This report synthesizes intelligence from three independent model analyses and a fallback summary. It highlights common findings, discrepancies, and operational implications.
+Combined Analysis:
+Gemini Analysis:
+Based on the provided documents, the Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution focused on achieving technological self-reliance and innovation in defence systems.
+Here's an overview of DRDO's activities and focus areas:
+**Research Laboratories:**
+*   **Aeronautical Development Establishment (ADE):** Specializes in aircraft and missile design.
+*   **Defence Electronics Research Laboratory (DERL):** Focuses on electronics and communications.
+*   **Mechanical Engineering Research Laboratory (MERL):** Works on ground systems and vehicles.
+*   **Naval Science and Technological Laboratory (NSTL):** Dedicated to submarine and ship technology.
+*   **Centre for Airborne Systems (CARS):** Develops avionics and mission systems.
+**Major Projects:**
+*   **FRCN:** A Fifth Generation Combat Aircraft project, incorporating stealth and AI-enabled capabilities.
+*   **ASTRA Missile:** An air-to-air missile featuring indigenous seekers and propulsion.
+*   **Lakshya Target:** An unmanned aerial vehicle used for training and reconnaissance.
+*   **Tactical Ballistic Missile (TBM):** A short-range precision strike system.
+**Advanced Technologies under Development:**
+*   **Directed Energy Weapons:** High-power laser and microwave systems.
+*   **Quantum Radar:** Detection systems utilizing quantum entanglement properties.
+*   **Additive
+Groq Analysis:
+Based on the provided context, the latest news related to DRDO (Defence Research and Development Organisation) includes:
+1. **Advanced Technologies**: DRDO is working on various advanced technologies such as Directed Energy Weapons, Quantum Radar, Additive Manufacturing, Artificial Intelligence, and Biotechnology.
+2. **Major Projects**: DRDO is involved in several major projects, including the development of the Fifth Generation Combat Aircraft (FRCN), ASTRA Missile, Lakshya Target, and Tactical Ballistic Missile (TBM).
+3. **Collaboration**: DRDO is collaborating with industry partners, academic institutions, and international organizations to accelerate the development of defence technologies.
+4. **Patents and Intellectual Property**: DRDO has filed over 400 patents in the last 5 years in critical defence technologies and is working on technology transfer to private industry for commercial applications.
+5. **Research Laboratories**: DRDO has several research laboratories, including the Aeronautical Development Establishment (ADE), Defence Electronics Research Laboratory (DERL), Mechanical Engineering Research Laboratory (MERL), Naval Science and Technological Laboratory (NSTL), and Centre for Airborne Systems (CARS).
+However, it's worth noting that the provided context does not include real-time news or updates. The information is based on the documents provided, which may not reflect the latest developments or news related to DRDO.
+If you're looking for the latest news on DRDO, I recommend checking reputable news sources or the official DRDO website for the most up-to-date information.
+Grok Analysis:
+No Grok output available.
+Fallback Analysis:
+Based on the retrieved documents:
+1. From 'Defence Research and Development: Innovation in Military Technology' (confidence: 35.8%):
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Developmen...
+2. From 'Document' (confidence: 34.5%):
+   The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile ...
+3. From 'Cybersecurity Strategy for Defence Installations 2023' (confidence: 13.2%):
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.
+Key Findings:
+- Gemini: Based on the provided documents, the Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution focused on achieving technological self-reliance and innovation in defence systems....
+- Groq: Based on the provided context, the latest news related to DRDO (Defence Research and Development Organisation) includes:...
+Detailed Analysis:
+Gemini Analysis:
+Based on the provided documents, the Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution focused on achieving technological self-reliance and innovation in defence systems.
+Here's an overview of DRDO's activities and focus areas:
+**Research Laboratories:**
+*   **Aeronautical Development Establishment (ADE):** Specializes in aircraft and missile design.
+*   **Defence Electronics Research Laboratory (DERL):** Focuses on electronics and communications.
+*   **Mechanical Engineering Research Laboratory (MERL):** Works on ground systems and vehicles.
+*   **Naval Science and Technological Laboratory (NSTL):** Dedicated to submarine and ship technology.
+*   **Centre for Airborne Systems (CARS):** Develops avionics and mission systems.
+**Major Projects:**
+*   **FRCN:** A Fifth Generation Combat Aircraft project, incorporating stealth and AI-enabled capabilities.
+*   **ASTRA Missile:** An air-to-air missile featuring indigenous seekers and propulsion.
+*   **Lakshya Target:** An unmanned aerial vehicle used for training and reconnaissance.
+*   **Tactical Ballistic Missile (TBM):** A short-range precision strike system.
+**Advanced Technologies under Development:**
+*   **Directed Energy Weapons:** High-power laser and microwave systems.
+*   **Quantum Radar:** Detection systems utilizing quantum entanglement properties.
+*   **Additive
+Groq Analysis:
+Based on the provided context, the latest news related to DRDO (Defence Research and Development Organisation) includes:
+1. **Advanced Technologies**: DRDO is working on various advanced technologies such as Directed Energy Weapons, Quantum Radar, Additive Manufacturing, Artificial Intelligence, and Biotechnology.
+2. **Major Projects**: DRDO is involved in several major projects, including the development of the Fifth Generation Combat Aircraft (FRCN), ASTRA Missile, Lakshya Target, and Tactical Ballistic Missile (TBM).
+3. **Collaboration**: DRDO is collaborating with industry partners, academic institutions, and international organizations to accelerate the development of defence technologies.
+4. **Patents and Intellectual Property**: DRDO has filed over 400 patents in the last 5 years in critical defence technologies and is working on technology transfer to private industry for commercial applications.
+5. **Research Laboratories**: DRDO has several research laboratories, including the Aeronautical Development Establishment (ADE), Defence Electronics Research Laboratory (DERL), Mechanical Engineering Research Laboratory (MERL), Naval Science and Technological Laboratory (NSTL), and Centre for Airborne Systems (CARS).
+However, it's worth noting that the provided context does not include real-time news or updates. The information is based on the documents provided, which may not reflect the latest developments or news related to DRDO.
+If you're looking for the latest news on DRDO, I recommend checking reputable news sources or the official DRDO website for the most up-to-date information.
+Grok Analysis:
+No Grok output available.
+Fallback Analysis:
+Based on the retrieved documents:
+1. From 'Defence Research and Development: Innovation in Military Technology' (confidence: 35.8%):
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Developmen...
+2. From 'Document' (confidence: 34.5%):
+   The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile ...
+3. From 'Cybersecurity Strategy for Defence Installations 2023' (confidence: 13.2%):
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat...
+Note: This is a summary from retrieved documents. For complete analysis, configure the Grok LLM API key.
+Retrieved Context and Sources:
+Document 1: Unknown Document
+Content: 
+        The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving 
+        technological self-reliance and innovation in defence systems.
+        Research Laboratories:
+        - Aeronautical Development Establishment (ADE): Aircraft and missile design
+        - Defence Electronics Research Laboratory (DERL): Electronics and communications
+        - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles
+        - Naval Science and Technological Laboratory (NSTL): Submarine and ship technology
+        - Centre for Airborne Systems (CARS): Avionics and mission systems
+        Major Projects:
+        - FRCN: Fifth Generation Combat Aircraft (stealth, AI-enabled)
+        - ASTRA Missile: Air-to-air missile with indigenous seekers and propulsion
+        - Lakshya Target: Unmanned aerial vehicle for training and reconnaissance
+        - Tactical Ballistic Missile (TBM): Short-range precision strike system
+        Advanced Technologies:
+        - Directed Energy Weapons: High-power laser and microwave systems
+        - Quantum Radar: Detection system using quantum entanglement properties
+        - Additive Manufacturing: 3D printing for complex defense components
+        - Artificial Intelligence: Machine learning for autonomous systems
+        - Biotechnology: Biological sensors and health monitoring systems
+        Collaboration:
+        - Industry partnerships with private sector for rapid development
+        - Academic collaborations with universities for research
+        - International partnerships with friendly nations for technology exchange
+        - Startup ecosystem fostering innovation in defense tech startups
+        Patents and Intellectual Property:
+        - Over 400 patents filed in last 5 years in critical defense technologies
+        - Technology transfer to private industry for commercial applications
+        - Open innovation platforms for crowd-sourced problem solving
+Relevance: 35.8%
+---
+Document 2: Defence Research and Development: Innovation in Military Technology
+Content: The Defence Research and Development Organisation (DRDO) is the premier R&amp;D institution driving technological self-reliance and innovation in defence systems Research Laboratories: - Aeronautical Development Establishment (ADE): Aircraft and missile design - Defence Electronics Research Laboratory (DERL): Electronics and communications - Mechanical Engineering Research Laboratory (MERL): Ground systems and vehicles - Naval Science and Technological Laboratory (NSTL): Submarine and ship technology - Centre for Airborne Systems (CARS): Avionics and mission systems Major Projects: - FRCN: Fifth Generation Combat Aircraft (stealth, AI-enabled) - ASTRA Missile: Air-to-air missile with indigenous seekers and propulsion - Lakshya Target: Unmanned aerial vehicle for training and reconnaissance - Tactical Ballistic Missile (TBM): Short-range precision strike system Advanced Technologies: - Directed Energy Weapons: High-power laser and microwave systems - Quantum Radar: Detection system using quantum entanglement properties - Additive Manufacturing: 3D printing for complex defense components - Artificial Intelligence: Machine learning for autonomous systems - Biotechnology: Biological sensors and health monitoring systems Collaboration: - Industry partnerships with private sector for rapid development - Academic collaborations with universities for research - International partnerships with friendly nations for technology exchange - Startup ecosystem fostering innovation in defense tech startups Patents and Intellectual Property: - Over 400 patents filed in last 5 years in critical defense technologies - Technology transfer to private industry for commercial applications - Open innovation platforms for crowd-sourced problem solving
+Relevance: 34.5%
+---
+Document 3: Unknown Document
+Content: 
+        The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, 
+        and information systems from cyber threats, both state-sponsored and non-state actors.
+        Threat Assessment:
+        - Nation-state adversaries targeting defence secrets and military capabilities
+        - Espionage activities targeting classified information and strategic plans
+        - Disruption attempts against operational command and control systems
+        - Theft of defense technology and intellectual property
+        Defensive Measures:
+        - Zero Trust Architecture: All access requires verification, no implicit trust
+        - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256)
+        - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens
+        - Air-Gapped Networks: Critical systems isolated from internet connectivity
+        - Continuous Monitoring: 24/7 intrusion detection and prevention systems
+        Operational Protocols:
+        - Defense Information Systems Agency (DISA) standards for network design
+        - Regular penetration testing by authorized ethical hackers (quarterly)
+        - Security incident response within 4 hours of detection
+        - Personnel security clearances updated annually with background verification
+        - Equipment procurement from certified vendors with security audits
+        Incident Response:
+        - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection
+        - Forensics preserved for investigation and prosecution
+        - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 13.2%
+---
+Document 4: Defence Budget Allocation 2023-24: Analysis and Distribution
+Content: The Defence Budget for 2023-24 has been allocated ₹1 72 lakh crores, representing 1 9% of GDP This allocation reflects the government's commitment to modernization and operational readiness Budget Distribution: - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance Key Allocations: - Army: ₹68,000 crores (40%) - Personnel, weapons, training - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems Major Projects Funded: - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years) - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores) - Rafale Production Line: 36 additional aircraft (₹8,000 crores) - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores) The budget supports approximately 1 3 million military and civilian personnel in the defence sector
+Relevance: 13.2%
+---
+Document 5: Unknown Document
+Content: 
+        This report details India's advanced weaponry systems currently in development or recently deployed, 
+        showcasing indigenous technological capabilities and international partnerships.
+        Missile Systems:
+        - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational
+        - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous
+        - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation
+        - PSLV/GSLV: Satellite launch systems with dual military applications
+        - Nirbhay: Subsonic cruise missile under development for extended range operations
+        Aircraft Systems:
+        - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems
+        - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades
+        - HAL Prachand: Indigenous light combat helicopter, 15 in operation
+        - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters
+        Naval Platforms:
+        - INS Vikramaditya: Carrier with integrated air defense and communications systems
+        - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion)
+        - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles
+        - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection
+        Ground Systems:
+        - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems
+        - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation
+        - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 13.0%
+---
+Document 6: Cybersecurity Strategy for Defence Installations 2023
+Content: The Defence Cybersecurity Strategy outlines measures to protect critical military infrastructure, communication networks, and information systems from cyber threats, both state-sponsored and non-state actors Threat Assessment: - Nation-state adversaries targeting defence secrets and military capabilities - Espionage activities targeting classified information and strategic plans - Disruption attempts against operational command and control systems - Theft of defense technology and intellectual property Defensive Measures: - Zero Trust Architecture: All access requires verification, no implicit trust - End-to-End Encryption: All sensitive communications use military-grade encryption (AES-256) - Multi-Factor Authentication: All personnel use biometric + password + hardware tokens - Air-Gapped Networks: Critical systems isolated from internet connectivity - Continuous Monitoring: 24/7 intrusion detection and prevention systems Operational Protocols: - Defense Information Systems Agency (DISA) standards for network design - Regular penetration testing by authorized ethical hackers (quarterly) - Security incident response within 4 hours of detection - Personnel security clearances updated annually with background verification - Equipment procurement from certified vendors with security audits Incident Response: - Cyber Incident Response Team (CIRT) activated within 15 minutes of threat detection - Forensics preserved for investigation and prosecution - Affected systems isolated within 30 minutes to prevent spread
+Relevance: 12.9%
+---
+Document 7: Unknown Document
+Content: 
+        The Defence Budget for 2023-24 has been allocated ₹1.72 lakh crores, representing 1.9% of GDP. 
+        This allocation reflects the government's commitment to modernization and operational readiness.
+        Budget Distribution:
+        - Capital Expenditure: ₹65,000 crores (38%) - New equipment, infrastructure, modernization
+        - Revenue Expenditure: ₹1,07,000 crores (62%) - Salaries, operations, maintenance
+        Key Allocations:
+        - Army: ₹68,000 crores (40%) - Personnel, weapons, training
+        - Navy: ₹35,000 crores (20%) - Maritime systems, submarines, aircraft carriers
+        - Air Force: ₹44,000 crores (25%) - Fighter jets, transport aircraft, air defense
+        - Strategic Forces: ₹25,000 crores (15%) - Nuclear deterrence, strategic systems
+        Major Projects Funded:
+        - Project 75-I: 6 Advanced Submarines (₹42,000 crores over 15 years)
+        - FRCN: Fifth Generation Combat Aircraft (₹15,000 crores)
+        - Rafale Production Line: 36 additional aircraft (₹8,000 crores)
+        - Indigenous Aircraft Carrier (INS Vikrant): ₹20,000 crores
+        - Missile Systems: BrahMos, Akash, QRSAM development (₹12,000 crores)
+        The budget supports approximately 1.3 million military and civilian personnel in the defence sector.
+Relevance: 12.8%
+---
+Document 8: Advanced Weaponry Systems: Development and Deployment
+Content: This report details India's advanced weaponry systems currently in development or recently deployed, showcasing indigenous technological capabilities and international partnerships Missile Systems: - BrahMos Cruise Missile: Hypersonic (Mach 3+), range 450 km, sea and land variants operational - Akash-NG Air Defence System: Multi-target engagement, range 30 km, fully indigenous - QRSAM: Quick Reaction Surface-to-Air Missile, range 25 km, autonomous operation - PSLV/GSLV: Satellite launch systems with dual military applications - Nirbhay: Subsonic cruise missile under development for extended range operations Aircraft Systems: - Rafale Fighter Jet: 36 aircraft on order from France, integration with indigenous systems - Tejas Light Combat Aircraft: 83 aircraft approved, 10 operational, with continuous upgrades - HAL Prachand: Indigenous light combat helicopter, 15 in operation - Transport Aircraft: C-17 Globemaster, C-130J Hercules, ALH utility helicopters Naval Platforms: - INS Vikramaditya: Carrier with integrated air defense and communications systems - Project 75-I Submarines: Advanced diesel-electric submarines with AIP (Air Independent Propulsion) - Guided Missile Destroyers: INS Kolkata-class, equipped with Brahmos missiles - Corvettes and Offshore Patrol Vessels: Coastal security and territorial waters protection Ground Systems: - T-72 Tank Upgrades: Enhanced armor, fire control, and engine systems - Arjun Main Battle Tank: Indigenous design, 118 tanks in operation - Combat Management Systems: Integrated battlefield network and decision support
+Relevance: 12.4%
+---
+Document 9: Unknown Document
+Content: 
+        India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast 
+        area with significant maritime trade routes and strategic importance.
+        Regional Challenges:
+        - Maritime disputes in South China Sea and Indian Ocean
+        - Terrorism and extremism affecting coastal security
+        - Piracy and armed robbery in key shipping lanes
+        - Unregulated arms trafficking and human trafficking
+        - Climate change impacts on island nations and maritime zones
+        Defence Partnerships:
+        - Quad Alliance: USA, Japan, Australia, India cooperation for peace and stability
+        - BIMSTEC: Bay of Bengal Initiative for regional security cooperation
+        - ASEAN Engagement: Strategic dialogue and military cooperation exercises
+        - Indian Ocean Rim Association: Coordination for maritime security
+        Operational Activities:
+        - Regular naval exercises: Malabar (USA, Japan, India), MILAN (regional navies)
+        - Joint air exercises with friendly nations to build interoperability
+        - Anti-piracy operations in Gulf of Aden and Indian Ocean
+        - Disaster relief and humanitarian assistance missions
+        Technology and Intelligence Sharing:
+        - Real-time information sharing on maritime threats and piracy
+        - Joint surveillance operations in critical sea lanes
+        - Coordinated response to emerging security threats
+        - Exchange of intelligence on terrorism and extremism funding
+        Future Strategy:
+        - Strengthening missile defense capabilities for regional credibility
+        - Expanding naval presence with additional carrier battle groups
+        - Building indigenous space-based surveillance and early warning systems
+        - Enhanced cyber defense for critical maritime and port infrastructure
+Relevance: 12.2%
+---
+Document 10: Indo-Pacific Security and Regional Defence Cooperation
+Content: India plays a crucial role in maintaining stability and security in the Indo-Pacific region, a geographically vast area with significant maritime trade routes and strategic importance Regional Challenges: - Maritime disputes in South China Sea and Indian Ocean - Terrorism and extremism affecting coastal security - Piracy and armed robbery in key shipping lanes - Unregulated arms trafficking and human trafficking - Climate change impacts on island nations and maritime zones Defence Partnerships: - Quad Alliance: USA, Japan, Australia, India cooperation for peace and stability - BIMSTEC: Bay of Bengal Initiative for regional security cooperation - ASEAN Engagement: Strategic dialogue and military cooperation exercises - Indian Ocean Rim Association: Coordination for maritime security Operational Activities: - Regular naval exercises: Malabar (USA, Japan, India), MILAN (regional navies) - Joint air exercises with friendly nations to build interoperability - Anti-piracy operations in Gulf of Aden and Indian Ocean - Disaster relief and humanitarian assistance missions Technology and Intelligence Sharing: - Real-time information sharing on maritime threats and piracy - Joint surveillance operations in critical sea lanes - Coordinated response to emerging security threats - Exchange of intelligence on terrorism and extremism funding Future Strategy: - Strengthening missile defense capabilities for regional credibility - Expanding naval presence with additional carrier battle groups - Building indigenous space-based surveillance and early warning systems - Enhanced cyber defense for critical maritime and port infrastructure
+Relevance: 12.1%
+---
+Document 11: Military Modernization Strategy: 2023-2035 Road Map
+Content: India's Military Modernization Strategy aims to create a technologically advanced, self-reliant defence force capable of addressing emerging security challenges in the Indo-Pacific region Strategic Pillars: 1 Technology Acquisition: Import of cutting-edge platforms with simultaneous indigenous development 2 Self-Reliance: 80% indigenous content in all new systems by 2030 3 Joint Operations: Enhanced interoperability between services through common C4I systems 4 Cybersecurity: Advanced cyber warfare capabilities and critical infrastructure protection 5 Space Applications: Military satellites for surveillance, navigation, and communication Priority Areas: - Hypersonic Missiles: Mach 5+ cruise missiles under development - 5G Networks: Military-grade 5G for unmanned systems and battlefield communication - AI Integration: Autonomous systems for surveillance and decision support - Quantum Computing: Encryption and cryptographic applications for secure communication - Artificial Intelligence: Machine learning for target identification and predictive maintenance Partnerships: - Technology partnerships with USA, France, Israel, Russia, and Japan - Co-development arrangements for systems like fighter jets and helicopters - Joint exercises and interoperability protocols with friendly nations Timeline: Capability goals set for 2025, 2028, 2032, and 2035 with measurable metrics
+Relevance: 11.4%
+---
+Document 12: Joint Theatre Command Implementation Roadmap
+Content: Implementation framework for establishing unified theatre commands as proposed by the Chief of Defence Staff This transformational reorganization consolidates geographical and functional commands under single theatre commander, creating streamlined command structures with unified planning and execution authorities Theatre commands include: Western Theatre (India-Pakistan border), Northern Theatre (China border, high altitude operations), Eastern Theatre (Bangladesh-Myanmar region), Maritime Theatre (Indian Ocean), Cyber Theatre (digital warfare operations), Space Theatre (satellite operations and space defence) Expected efficiency gains from unification: 15-20% reduction in administrative overhead and redundant support structures, faster decision-making cycles through simplified command chains, improved inter-service coordination eliminating compartmentalization, and better resource optimization Transition timeline structured in three phases: Phase 1 (2024-25) establishes new command structures with compatible organizational frameworks; Phase 2 (2025-26) implements resource consolidation with integrated logistics and personnel management; Phase 3 (2026-27) achieves full operationalization with theatre-level integrated exercises demonstrating seamless inter-service coordination Risk mitigation strategies address potential institutional disruption through: smooth transition protocols minimizing operational gaps, comprehensive training programs for officers and support staff adapting to new command structures, maintenance of continuity during transition period, and retention mechanisms for experienced personnel Technology integration includes unified command and control systems, real-time data sharing across services, and AI-based decision support systems providing situational assessment and recommendation synthesis Performance metrics for successful theatre command implementation include reduced decision-making timelines, improved operational effectiveness metrics, enhanced inter-service coordination demonstrated through joint exercises, and cost optimization targets The transformation represents major institutional change requiring sustained commitment from military leadership, government support, and international partnerships with allied nations having similar structures
+Relevance: 11.0%
+---
+Document 13: Cyber Defence Architecture and National Digital Resilience Plan
+Content: Multi-layered cyber defence architecture protects critical defence infrastructure, government networks, and national security installations against sophisticated cyber attacks Establishment of National Cyber Security Centre with 24/7 monitoring capabilities provides continuous threat detection, rapid response activation, and incident management Threat detection capabilities target nation-state level attacks, organized cyber criminal groups, and individual hackers, with machine learning systems identifying novel attack patterns and zero-day exploits Integration with civil agencies including CERT-In, intelligence agencies, and critical infrastructure operators creates coordinated response mechanisms The architecture incorporates multiple security layers: perimeter defence with advanced firewalls and intrusion detection systems, internal segmentation isolating critical systems, endpoint protection on all connected devices, and application-level security Training of 10,000 cyber warriors annually builds indigenous cyber workforce capability reducing dependence on foreign expertise Investment in indigenous cybersecurity solutions reduces vendor dependency and protects sensitive military information from potential backdoors in foreign software Collaboration with academia establishes cyber research centers, develops advanced security technologies, and creates talent pipeline for continuous workforce expansion Cyber defence budget allocation of ₹5,000 crores over 5 years supports infrastructure development, training programs, and advanced technology acquisition Specific focus areas include: encryption system development ensuring unhackable communications, AI-based intrusion detection identifying sophisticated attacks, quantum computing preparation developing post-quantum cryptography, and supply chain security ensuring no compromised components enter defence systems International partnerships with allied nations strengthen collective cyber defence posture through information sharing and coordinated response protocols Offensive cyber capabilities provide deterrence and retaliatory options against hostile cyber operations Regular cyber war games and simulation exercises maintain readiness and identify capability gaps
+Relevance: 10.9%
+---
+Document 14: Cyber Defence Architecture and National Dig</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>multi-model-synthesis</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>18.07613134384155</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>